<commit_message>
Cap nhat cac doan ly do
</commit_message>
<xml_diff>
--- a/NguyenTienPhat_Day22_model.xlsx
+++ b/NguyenTienPhat_Day22_model.xlsx
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="B27" s="14">
-        <f>'2_Pricing'!$B$95</f>
+        <f>'2_Pricing'!$B$96</f>
         <v>0.03787170779220779</v>
       </c>
       <c r="C27" s="15" t="inlineStr">
@@ -1124,7 +1124,7 @@
         </is>
       </c>
       <c r="B28" s="14">
-        <f>'2_Pricing'!$B$96</f>
+        <f>'2_Pricing'!$B$97</f>
         <v>0.11361512337662337</v>
       </c>
       <c r="C28" s="15" t="inlineStr">
@@ -1144,7 +1144,7 @@
         </is>
       </c>
       <c r="B29" s="14">
-        <f>'2_Pricing'!$B$97</f>
+        <f>'2_Pricing'!$B$98</f>
         <v>0.12417582417582418</v>
       </c>
       <c r="C29" s="15" t="inlineStr">
@@ -1164,7 +1164,7 @@
         </is>
       </c>
       <c r="B30" s="17">
-        <f>'2_Pricing'!$B$98</f>
+        <f>'2_Pricing'!$B$99</f>
         <v>0.6950154505229285</v>
       </c>
       <c r="C30" s="15" t="inlineStr">
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="B31" s="17">
-        <f>'2_Pricing'!$B$99</f>
+        <f>'2_Pricing'!$B$100</f>
         <v>0.5746102958015268</v>
       </c>
       <c r="C31" s="15" t="inlineStr">
@@ -1208,7 +1208,7 @@
         </is>
       </c>
       <c r="B32" s="19">
-        <f>'2_Pricing'!$B$100</f>
+        <f>'2_Pricing'!$B$101</f>
         <v>0.8</v>
       </c>
       <c r="C32" s="15" t="inlineStr">
@@ -1228,7 +1228,7 @@
         </is>
       </c>
       <c r="B33" s="20">
-        <f>'4_Channel_Fit'!$B$45</f>
+        <f>'4_Channel_Fit'!$B$46</f>
         <v>538.5376862337663</v>
       </c>
       <c r="C33" s="15" t="inlineStr">
@@ -1248,7 +1248,7 @@
         </is>
       </c>
       <c r="B34" s="21">
-        <f>'4_Channel_Fit'!$B$46</f>
+        <f>'4_Channel_Fit'!$B$47</f>
         <v>2.5811209439528024</v>
       </c>
       <c r="C34" s="15" t="inlineStr">
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="B40" s="22" t="str">
-        <f>IF(AND('2_Pricing'!$B$37&gt;='2_Pricing'!$B$7,'2_Pricing'!$B$47&gt;='2_Pricing'!$B$44,'2_Pricing'!$B$47&lt;=0.85),"✓ Giá ≥ giá sàn và GM trong vùng 60–85%","✗ Chưa đạt: xem 2_Pricing mục A và D")</f>
+        <f>IF(AND('2_Pricing'!$B$38&gt;='2_Pricing'!$B$7,'2_Pricing'!$B$48&gt;='2_Pricing'!$B$45,'2_Pricing'!$B$48&lt;=0.85),"✓ Giá ≥ giá sàn và GM trong vùng 60–85%","✗ Chưa đạt: xem 2_Pricing mục A và D")</f>
         <v>✓ Giá ≥ giá sàn và GM trong vùng 60–85%</v>
       </c>
       <c r="C40" s="7" t="n"/>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="B41" s="22" t="str">
-        <f>IF(AND(ISNUMBER('2_Pricing'!$B$63),ISNUMBER('2_Pricing'!$B$64)),"✓ Breakeven "&amp;ROUND('2_Pricing'!$B$63*100,1)&amp;"% so với "&amp;ROUND('2_Pricing'!$B$64*100,1)&amp;"% (eval hiện tại là ước tính, chưa đo)","✗ Thiếu")</f>
+        <f>IF(AND(ISNUMBER('2_Pricing'!$B$64),ISNUMBER('2_Pricing'!$B$65)),"✓ Breakeven "&amp;ROUND('2_Pricing'!$B$64*100,1)&amp;"% so với "&amp;ROUND('2_Pricing'!$B$65*100,1)&amp;"% (eval hiện tại là ước tính, chưa đo)","✗ Thiếu")</f>
         <v>✓ Breakeven 57.5% so với 80% (eval hiện tại là ước tính, chưa đo)</v>
       </c>
       <c r="C41" s="7" t="n"/>
@@ -2628,16 +2628,15 @@
       <c r="F63" s="4" t="n"/>
       <c r="G63" s="4" t="n"/>
     </row>
-    <row r="64" ht="42.5" customHeight="1">
+    <row r="64" ht="56" customHeight="1">
       <c r="A64" s="18" t="inlineStr">
         <is>
           <t>Biến thể đã chọn và 1 câu lý do</t>
         </is>
       </c>
-      <c r="B64" s="25" t="inlineStr">
-        <is>
-          <t>Biến thể A: ca AI không chắc được đưa vào hàng đợi duyệt trong sản phẩm cho kế toán của khách (khách tự xử lý, như Intercom Fin escalate sang agent của khách), nên không vào COGS; COGS chỉ gánh QA nội bộ lấy mẫu. Cột Biến thể B bên dưới cho thấy Cost/Job nếu bạn phải giao kết quả.</t>
-        </is>
+      <c r="B64" s="25" t="str">
+        <f>"Tôi chọn Biến thể A: hóa đơn nào AI không chắc sẽ chuyển cho kế toán của khách duyệt ngay trong sản phẩm, nên công của họ không tính vào chi phí của tôi. Tôi chỉ tốn tiền cho phần kiểm tra mẫu "&amp;ROUND($B$68*100,0)&amp;"%. Nếu tôi phải tự xử lý các ca đó (Biến thể B), Cost/Job tăng lên $"&amp;ROUND($C$88,3)&amp;" và lãi gộp chỉ còn "&amp;ROUND('2_Pricing'!$B$47*100,0)&amp;"%, nên tôi không bán theo cách này."</f>
+        <v>Tôi chọn Biến thể A: hóa đơn nào AI không chắc sẽ chuyển cho kế toán của khách duyệt ngay trong sản phẩm, nên công của họ không tính vào chi phí của tôi. Tôi chỉ tốn tiền cho phần kiểm tra mẫu 4%. Nếu tôi phải tự xử lý các ca đó (Biến thể B), Cost/Job tăng lên $0.103 và lãi gộp chỉ còn 17%, nên tôi không bán theo cách này.</v>
       </c>
       <c r="C64" s="7" t="n"/>
       <c r="D64" s="7" t="n"/>
@@ -3426,7 +3425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G100"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -3877,10 +3876,9 @@
           <t>Lý do chọn neo</t>
         </is>
       </c>
-      <c r="B25" s="25" t="inlineStr">
-        <is>
-          <t>Khách tự kiểm chứng được lương nhân viên (số trên bảng lương), còn "giá trị tạo ra" phải tin vào ước tính của nhà cung cấp. Lưu ý: neo giá trị cho giá trần THẤP HƠN giá sàn, tức là ở mức lương Việt Nam, đòn bẩy giảm Cost/Job (xem bảng model bên dưới) quan trọng hơn chuyện tăng giá.</t>
-        </is>
+      <c r="B25" s="25" t="str">
+        <f>"Tôi neo giá theo lương người nhập liệu vì khách tự kiểm tra được con số này trên bảng lương của họ. ""Giá trị AI tạo ra"" thì họ phải tin vào ước tính của tôi. Giá đề xuất "&amp;ROUND($B$37,0)&amp;" đ/hóa đơn rẻ hơn thuê người khoảng "&amp;ROUND($B$40*100,0)&amp;"%, nằm giữa giá sàn ("&amp;ROUND($B$8,0)&amp;" đ) và giá trần ("&amp;ROUND($B$27,0)&amp;" đ)."</f>
+        <v>Tôi neo giá theo lương người nhập liệu vì khách tự kiểm tra được con số này trên bảng lương của họ. "Giá trị AI tạo ra" thì họ phải tin vào ước tính của tôi. Giá đề xuất 3260 đ/hóa đơn rẻ hơn thuê người khoảng 58%, nằm giữa giá sàn (2982 đ) và giá trần (5385 đ).</v>
       </c>
       <c r="C25" s="7" t="n"/>
       <c r="D25" s="7" t="n"/>
@@ -3888,39 +3886,27 @@
       <c r="F25" s="7" t="n"/>
       <c r="G25" s="8" t="n"/>
     </row>
-    <row r="26" ht="15.5" customHeight="1">
-      <c r="A26" s="13" t="inlineStr">
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="26" t="inlineStr"/>
+      <c r="B26" s="27" t="inlineStr">
+        <is>
+          <t>Lưu ý: neo giá trị cho giá trần THẤP HƠN giá sàn, nên đòn bẩy giảm Cost/Job (bảng model ở mục G) quan trọng hơn chuyện tăng giá.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15.5" customHeight="1">
+      <c r="A27" s="13" t="inlineStr">
         <is>
           <t>GIÁ TRẦN (theo neo đã chọn, cận trên)</t>
         </is>
       </c>
-      <c r="B26" s="41">
+      <c r="B27" s="41">
         <f>IF($B$24="Nhân công",$B$17,$B$22)</f>
         <v>5384.615384615385</v>
       </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="C27" s="15" t="inlineStr">
         <is>
           <t>VND / job</t>
-        </is>
-      </c>
-      <c r="D26" s="16" t="inlineStr"/>
-      <c r="E26" s="7" t="n"/>
-      <c r="F26" s="7" t="n"/>
-      <c r="G26" s="8" t="n"/>
-    </row>
-    <row r="27" ht="15.5" customHeight="1">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>Giá trần quy đổi</t>
-        </is>
-      </c>
-      <c r="B27" s="32">
-        <f>$B$26/'1_Cost_Job'!$B$5</f>
-        <v>0.20512820512820512</v>
-      </c>
-      <c r="C27" s="15" t="inlineStr">
-        <is>
-          <t>$ / job</t>
         </is>
       </c>
       <c r="D27" s="16" t="inlineStr"/>
@@ -3928,57 +3914,58 @@
       <c r="F27" s="7" t="n"/>
       <c r="G27" s="8" t="n"/>
     </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+    <row r="28" ht="15.5" customHeight="1">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>Giá trần quy đổi</t>
+        </is>
+      </c>
+      <c r="B28" s="32">
+        <f>$B$27/'1_Cost_Job'!$B$5</f>
+        <v>0.20512820512820512</v>
+      </c>
+      <c r="C28" s="15" t="inlineStr">
+        <is>
+          <t>$ / job</t>
+        </is>
+      </c>
+      <c r="D28" s="16" t="inlineStr"/>
+      <c r="E28" s="7" t="n"/>
+      <c r="F28" s="7" t="n"/>
+      <c r="G28" s="8" t="n"/>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>C. Giá bán đề xuất — Hybrid (phí nền + theo hóa đơn hoàn thành vượt gói)</t>
         </is>
       </c>
-      <c r="B29" s="4" t="n"/>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="n"/>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="n"/>
-      <c r="G29" s="4" t="n"/>
-    </row>
-    <row r="30" ht="29" customHeight="1">
-      <c r="A30" s="18" t="inlineStr">
+      <c r="B30" s="4" t="n"/>
+      <c r="C30" s="4" t="n"/>
+      <c r="D30" s="4" t="n"/>
+      <c r="E30" s="4" t="n"/>
+      <c r="F30" s="4" t="n"/>
+      <c r="G30" s="4" t="n"/>
+    </row>
+    <row r="31" ht="29" customHeight="1">
+      <c r="A31" s="18" t="inlineStr">
         <is>
           <t>Phí nền / tháng</t>
         </is>
       </c>
-      <c r="B30" s="23" t="n">
+      <c r="B31" s="23" t="n">
         <v>1100000</v>
       </c>
-      <c r="C30" s="15" t="inlineStr">
+      <c r="C31" s="15" t="inlineStr">
         <is>
           <t>VND / khách</t>
         </is>
       </c>
-      <c r="D30" s="16" t="inlineStr">
+      <c r="D31" s="16" t="inlineStr">
         <is>
           <t>Đổi lấy thứ cụ thể: kết nối phần mềm kế toán + SLA xử lý trong ngày + hạn mức hóa đơn trong gói.</t>
         </is>
       </c>
-      <c r="E30" s="7" t="n"/>
-      <c r="F30" s="7" t="n"/>
-      <c r="G30" s="8" t="n"/>
-    </row>
-    <row r="31" ht="15.5" customHeight="1">
-      <c r="A31" s="18" t="inlineStr">
-        <is>
-          <t>Số hóa đơn hoàn thành gồm trong gói</t>
-        </is>
-      </c>
-      <c r="B31" s="23" t="n">
-        <v>350</v>
-      </c>
-      <c r="C31" s="15" t="inlineStr">
-        <is>
-          <t>hóa đơn</t>
-        </is>
-      </c>
-      <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="7" t="n"/>
       <c r="F31" s="7" t="n"/>
       <c r="G31" s="8" t="n"/>
@@ -3986,22 +3973,18 @@
     <row r="32" ht="15.5" customHeight="1">
       <c r="A32" s="18" t="inlineStr">
         <is>
-          <t>Giá mỗi hóa đơn hoàn thành vượt gói</t>
+          <t>Số hóa đơn hoàn thành gồm trong gói</t>
         </is>
       </c>
       <c r="B32" s="23" t="n">
-        <v>3500</v>
+        <v>350</v>
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>VND / job</t>
-        </is>
-      </c>
-      <c r="D32" s="16" t="inlineStr">
-        <is>
-          <t>Chỉ tính hóa đơn HOÀN THÀNH theo định nghĩa job ở 1_Cost_Job S1.</t>
-        </is>
-      </c>
+          <t>hóa đơn</t>
+        </is>
+      </c>
+      <c r="D32" s="16" t="inlineStr"/>
       <c r="E32" s="7" t="n"/>
       <c r="F32" s="7" t="n"/>
       <c r="G32" s="8" t="n"/>
@@ -4009,20 +3992,20 @@
     <row r="33" ht="15.5" customHeight="1">
       <c r="A33" s="18" t="inlineStr">
         <is>
-          <t>Hóa đơn hoàn thành / khách / tháng (điển hình)</t>
+          <t>Giá mỗi hóa đơn hoàn thành vượt gói</t>
         </is>
       </c>
       <c r="B33" s="23" t="n">
-        <v>520</v>
+        <v>3500</v>
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>job</t>
+          <t>VND / job</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>= 650 hóa đơn thử × containment 80%. GIẢ ĐỊNH, cần xác minh với khách pilot.</t>
+          <t>Chỉ tính hóa đơn HOÀN THÀNH theo định nghĩa job ở 1_Cost_Job S1.</t>
         </is>
       </c>
       <c r="E33" s="7" t="n"/>
@@ -4032,19 +4015,22 @@
     <row r="34" ht="15.5" customHeight="1">
       <c r="A34" s="18" t="inlineStr">
         <is>
-          <t>Doanh thu / khách / tháng</t>
-        </is>
-      </c>
-      <c r="B34" s="29">
-        <f>$B$30+MAX(0,$B$33-$B$31)*$B$32</f>
-        <v>1695000.0</v>
+          <t>Hóa đơn hoàn thành / khách / tháng (điển hình)</t>
+        </is>
+      </c>
+      <c r="B34" s="23" t="n">
+        <v>520</v>
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>VND</t>
-        </is>
-      </c>
-      <c r="D34" s="16" t="inlineStr"/>
+          <t>job</t>
+        </is>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>= 650 hóa đơn thử × containment 80%. GIẢ ĐỊNH, cần xác minh với khách pilot.</t>
+        </is>
+      </c>
       <c r="E34" s="7" t="n"/>
       <c r="F34" s="7" t="n"/>
       <c r="G34" s="8" t="n"/>
@@ -4052,23 +4038,19 @@
     <row r="35" ht="15.5" customHeight="1">
       <c r="A35" s="18" t="inlineStr">
         <is>
-          <t>ARPU / tháng</t>
-        </is>
-      </c>
-      <c r="B35" s="20">
-        <f>$B$34/'1_Cost_Job'!$B$5</f>
-        <v>64.57142857142857</v>
+          <t>Doanh thu / khách / tháng</t>
+        </is>
+      </c>
+      <c r="B35" s="29">
+        <f>$B$31+MAX(0,$B$34-$B$32)*$B$33</f>
+        <v>1695000.0</v>
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>$ / tháng</t>
-        </is>
-      </c>
-      <c r="D35" s="16" t="inlineStr">
-        <is>
-          <t>Dùng cho 4_Channel_Fit.</t>
-        </is>
-      </c>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr"/>
       <c r="E35" s="7" t="n"/>
       <c r="F35" s="7" t="n"/>
       <c r="G35" s="8" t="n"/>
@@ -4076,36 +4058,40 @@
     <row r="36" ht="15.5" customHeight="1">
       <c r="A36" s="18" t="inlineStr">
         <is>
-          <t>Giá hiệu dụng / job hoàn thành</t>
-        </is>
-      </c>
-      <c r="B36" s="29">
-        <f>$B$34/$B$33</f>
-        <v>3259.6153846153848</v>
+          <t>ARPU / tháng</t>
+        </is>
+      </c>
+      <c r="B36" s="20">
+        <f>$B$35/'1_Cost_Job'!$B$5</f>
+        <v>64.57142857142857</v>
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>VND / job</t>
-        </is>
-      </c>
-      <c r="D36" s="16" t="inlineStr"/>
+          <t>$ / tháng</t>
+        </is>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>Dùng cho 4_Channel_Fit.</t>
+        </is>
+      </c>
       <c r="E36" s="7" t="n"/>
       <c r="F36" s="7" t="n"/>
       <c r="G36" s="8" t="n"/>
     </row>
     <row r="37" ht="15.5" customHeight="1">
-      <c r="A37" s="13" t="inlineStr">
-        <is>
-          <t>GIÁ BÁN ĐỀ XUẤT (hiệu dụng)</t>
-        </is>
-      </c>
-      <c r="B37" s="14">
-        <f>$B$36/'1_Cost_Job'!$B$5</f>
-        <v>0.12417582417582418</v>
+      <c r="A37" s="18" t="inlineStr">
+        <is>
+          <t>Giá hiệu dụng / job hoàn thành</t>
+        </is>
+      </c>
+      <c r="B37" s="29">
+        <f>$B$35/$B$34</f>
+        <v>3259.6153846153848</v>
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>$ / job</t>
+          <t>VND / job</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
@@ -4114,18 +4100,18 @@
       <c r="G37" s="8" t="n"/>
     </row>
     <row r="38" ht="15.5" customHeight="1">
-      <c r="A38" s="18" t="inlineStr">
-        <is>
-          <t>Hóa đơn thử / khách / tháng</t>
-        </is>
-      </c>
-      <c r="B38" s="29">
-        <f>$B$33/'1_Cost_Job'!$B$22</f>
-        <v>650.0</v>
+      <c r="A38" s="13" t="inlineStr">
+        <is>
+          <t>GIÁ BÁN ĐỀ XUẤT (hiệu dụng)</t>
+        </is>
+      </c>
+      <c r="B38" s="14">
+        <f>$B$37/'1_Cost_Job'!$B$5</f>
+        <v>0.12417582417582418</v>
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>job</t>
+          <t>$ / job</t>
         </is>
       </c>
       <c r="D38" s="16" t="inlineStr"/>
@@ -4136,39 +4122,43 @@
     <row r="39" ht="15.5" customHeight="1">
       <c r="A39" s="18" t="inlineStr">
         <is>
-          <t>Rẻ hơn thuê người</t>
-        </is>
-      </c>
-      <c r="B39" s="19">
-        <f>1-$B$36/$B$13</f>
-        <v>0.5762499999999999</v>
+          <t>Hóa đơn thử / khách / tháng</t>
+        </is>
+      </c>
+      <c r="B39" s="29">
+        <f>$B$34/'1_Cost_Job'!$B$22</f>
+        <v>650.0</v>
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D39" s="16" t="inlineStr">
-        <is>
-          <t>Đây là câu trả lời cho khách: so với lương nhân viên.</t>
-        </is>
-      </c>
+          <t>job</t>
+        </is>
+      </c>
+      <c r="D39" s="16" t="inlineStr"/>
       <c r="E39" s="7" t="n"/>
       <c r="F39" s="7" t="n"/>
       <c r="G39" s="8" t="n"/>
     </row>
-    <row r="40" ht="29" customHeight="1">
+    <row r="40" ht="15.5" customHeight="1">
       <c r="A40" s="18" t="inlineStr">
         <is>
-          <t>Giá ≥ giá sàn (3 × Cost/Job)?</t>
-        </is>
-      </c>
-      <c r="B40" s="22" t="str">
-        <f>IF($B$37&gt;=$B$7,"✓ Giá đề xuất ≥ giá sàn","✗ Giá đề xuất &lt; giá sàn — quay lại Tab 1, đừng sửa giá cho đẹp")</f>
-        <v>✓ Giá đề xuất ≥ giá sàn</v>
-      </c>
-      <c r="C40" s="7" t="n"/>
-      <c r="D40" s="7" t="n"/>
+          <t>Rẻ hơn thuê người</t>
+        </is>
+      </c>
+      <c r="B40" s="19">
+        <f>1-$B$37/$B$13</f>
+        <v>0.5762499999999999</v>
+      </c>
+      <c r="C40" s="15" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>Đây là câu trả lời cho khách: so với lương nhân viên.</t>
+        </is>
+      </c>
       <c r="E40" s="7" t="n"/>
       <c r="F40" s="7" t="n"/>
       <c r="G40" s="8" t="n"/>
@@ -4176,12 +4166,12 @@
     <row r="41" ht="29" customHeight="1">
       <c r="A41" s="18" t="inlineStr">
         <is>
-          <t>Giá ≤ giá trần?</t>
+          <t>Giá ≥ giá sàn (3 × Cost/Job)?</t>
         </is>
       </c>
       <c r="B41" s="22" t="str">
-        <f>IF($B$37&lt;=$B$27,"✓ Giá đề xuất nằm trong vùng giá bán (sàn → trần)","~ Giá đề xuất vượt giá trần theo neo đã chọn")</f>
-        <v>✓ Giá đề xuất nằm trong vùng giá bán (sàn → trần)</v>
+        <f>IF($B$38&gt;=$B$7,"✓ Giá đề xuất ≥ giá sàn","✗ Giá đề xuất &lt; giá sàn — quay lại Tab 1, đừng sửa giá cho đẹp")</f>
+        <v>✓ Giá đề xuất ≥ giá sàn</v>
       </c>
       <c r="C41" s="7" t="n"/>
       <c r="D41" s="7" t="n"/>
@@ -4189,58 +4179,54 @@
       <c r="F41" s="7" t="n"/>
       <c r="G41" s="8" t="n"/>
     </row>
-    <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="3" t="inlineStr">
+    <row r="42" ht="29" customHeight="1">
+      <c r="A42" s="18" t="inlineStr">
+        <is>
+          <t>Giá ≤ giá trần?</t>
+        </is>
+      </c>
+      <c r="B42" s="22" t="str">
+        <f>IF($B$38&lt;=$B$28,"✓ Giá đề xuất nằm trong vùng giá bán (sàn → trần)","~ Giá đề xuất vượt giá trần theo neo đã chọn")</f>
+        <v>✓ Giá đề xuất nằm trong vùng giá bán (sàn → trần)</v>
+      </c>
+      <c r="C42" s="7" t="n"/>
+      <c r="D42" s="7" t="n"/>
+      <c r="E42" s="7" t="n"/>
+      <c r="F42" s="7" t="n"/>
+      <c r="G42" s="8" t="n"/>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>D. Gross Margin</t>
         </is>
       </c>
-      <c r="B43" s="4" t="n"/>
-      <c r="C43" s="4" t="n"/>
-      <c r="D43" s="4" t="n"/>
-      <c r="E43" s="4" t="n"/>
-      <c r="F43" s="4" t="n"/>
-      <c r="G43" s="4" t="n"/>
-    </row>
-    <row r="44" ht="15.5" customHeight="1">
-      <c r="A44" s="18" t="inlineStr">
-        <is>
-          <t>Mục tiêu GM</t>
-        </is>
-      </c>
-      <c r="B44" s="28" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="C44" s="15" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D44" s="16" t="inlineStr">
-        <is>
-          <t>Dưới 50% là vùng nguy hiểm; trên 85% gần như chắc chắn là quên chi phí.</t>
-        </is>
-      </c>
-      <c r="E44" s="7" t="n"/>
-      <c r="F44" s="7" t="n"/>
-      <c r="G44" s="8" t="n"/>
+      <c r="B44" s="4" t="n"/>
+      <c r="C44" s="4" t="n"/>
+      <c r="D44" s="4" t="n"/>
+      <c r="E44" s="4" t="n"/>
+      <c r="F44" s="4" t="n"/>
+      <c r="G44" s="4" t="n"/>
     </row>
     <row r="45" ht="15.5" customHeight="1">
       <c r="A45" s="18" t="inlineStr">
         <is>
-          <t>GM — Biến thể A</t>
-        </is>
-      </c>
-      <c r="B45" s="19">
-        <f>1-'1_Cost_Job'!$B$88/$B$37</f>
-        <v>0.6950154505229285</v>
+          <t>Mục tiêu GM</t>
+        </is>
+      </c>
+      <c r="B45" s="28" t="n">
+        <v>0.6</v>
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D45" s="16" t="inlineStr"/>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>Dưới 50% là vùng nguy hiểm; trên 85% gần như chắc chắn là quên chi phí.</t>
+        </is>
+      </c>
       <c r="E45" s="7" t="n"/>
       <c r="F45" s="7" t="n"/>
       <c r="G45" s="8" t="n"/>
@@ -4248,59 +4234,63 @@
     <row r="46" ht="15.5" customHeight="1">
       <c r="A46" s="18" t="inlineStr">
         <is>
-          <t>GM — Biến thể B</t>
+          <t>GM — Biến thể A</t>
         </is>
       </c>
       <c r="B46" s="19">
-        <f>1-'1_Cost_Job'!$C$88/$B$37</f>
-        <v>0.17208705148833459</v>
+        <f>1-'1_Cost_Job'!$B$88/$B$38</f>
+        <v>0.6950154505229285</v>
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D46" s="16" t="inlineStr">
-        <is>
-          <t>Cho thấy chọn sai biến thể → Cost/Job sai vài lần.</t>
-        </is>
-      </c>
+      <c r="D46" s="16" t="inlineStr"/>
       <c r="E46" s="7" t="n"/>
       <c r="F46" s="7" t="n"/>
       <c r="G46" s="8" t="n"/>
     </row>
     <row r="47" ht="15.5" customHeight="1">
-      <c r="A47" s="13" t="inlineStr">
-        <is>
-          <t>GROSS MARGIN — biến thể đang chọn</t>
-        </is>
-      </c>
-      <c r="B47" s="17">
-        <f>IF('1_Cost_Job'!$B$8="A",$B$45,$B$46)</f>
-        <v>0.6950154505229285</v>
+      <c r="A47" s="18" t="inlineStr">
+        <is>
+          <t>GM — Biến thể B</t>
+        </is>
+      </c>
+      <c r="B47" s="19">
+        <f>1-'1_Cost_Job'!$C$88/$B$38</f>
+        <v>0.17208705148833459</v>
       </c>
       <c r="C47" s="15" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D47" s="16" t="inlineStr"/>
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>Cho thấy chọn sai biến thể → Cost/Job sai vài lần.</t>
+        </is>
+      </c>
       <c r="E47" s="7" t="n"/>
       <c r="F47" s="7" t="n"/>
       <c r="G47" s="8" t="n"/>
     </row>
-    <row r="48" ht="29" customHeight="1">
-      <c r="A48" s="18" t="inlineStr">
-        <is>
-          <t>Đánh giá GM</t>
-        </is>
-      </c>
-      <c r="B48" s="22" t="str">
-        <f>IF($B$47&gt;0.85,"✗ GM &gt; 85%: gần như chắc chắn quên một khoản chi phí",IF($B$47&gt;=$B$44,"✓ GM đạt mục tiêu ≥ 60%",IF($B$47&gt;=0.5,"~ GM 50–60%: cần kế hoạch cải thiện","✗ GM &lt; 50%: vùng nguy hiểm")))</f>
-        <v>✓ GM đạt mục tiêu ≥ 60%</v>
-      </c>
-      <c r="C48" s="7" t="n"/>
-      <c r="D48" s="7" t="n"/>
+    <row r="48" ht="15.5" customHeight="1">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>GROSS MARGIN — biến thể đang chọn</t>
+        </is>
+      </c>
+      <c r="B48" s="17">
+        <f>IF('1_Cost_Job'!$B$8="A",$B$46,$B$47)</f>
+        <v>0.6950154505229285</v>
+      </c>
+      <c r="C48" s="15" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr"/>
       <c r="E48" s="7" t="n"/>
       <c r="F48" s="7" t="n"/>
       <c r="G48" s="8" t="n"/>
@@ -4308,42 +4298,38 @@
     <row r="49" ht="29" customHeight="1">
       <c r="A49" s="18" t="inlineStr">
         <is>
-          <t>Phí cổng thanh toán (ước tính, chưa đưa vào Cost/Job)</t>
-        </is>
-      </c>
-      <c r="B49" s="28" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="C49" s="15" t="inlineStr">
-        <is>
-          <t>% doanh thu</t>
-        </is>
-      </c>
-      <c r="D49" s="16" t="inlineStr">
-        <is>
-          <t>Từ vòng phản biện (Prompt_Log.md, 4.7.1): khoản này chưa nằm trong 5 thành phần của đề. ƯỚC TÍNH, chưa xác minh với cổng thanh toán.</t>
-        </is>
-      </c>
+          <t>Đánh giá GM</t>
+        </is>
+      </c>
+      <c r="B49" s="22" t="str">
+        <f>IF($B$48&gt;0.85,"✗ GM &gt; 85%: gần như chắc chắn quên một khoản chi phí",IF($B$48&gt;=$B$45,"✓ GM đạt mục tiêu ≥ 60%",IF($B$48&gt;=0.5,"~ GM 50–60%: cần kế hoạch cải thiện","✗ GM &lt; 50%: vùng nguy hiểm")))</f>
+        <v>✓ GM đạt mục tiêu ≥ 60%</v>
+      </c>
+      <c r="C49" s="7" t="n"/>
+      <c r="D49" s="7" t="n"/>
       <c r="E49" s="7" t="n"/>
       <c r="F49" s="7" t="n"/>
       <c r="G49" s="8" t="n"/>
     </row>
-    <row r="50" ht="15.5" customHeight="1">
+    <row r="50" ht="29" customHeight="1">
       <c r="A50" s="18" t="inlineStr">
         <is>
-          <t>GM sau phí cổng thanh toán</t>
-        </is>
-      </c>
-      <c r="B50" s="19">
-        <f>$B$47-$B$49</f>
-        <v>0.6700154505229284</v>
+          <t>Phí cổng thanh toán (ước tính, chưa đưa vào Cost/Job)</t>
+        </is>
+      </c>
+      <c r="B50" s="28" t="n">
+        <v>0.025</v>
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D50" s="16" t="inlineStr"/>
+          <t>% doanh thu</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>Từ vòng phản biện (Prompt_Log.md, 4.7.1): khoản này chưa nằm trong 5 thành phần của đề. ƯỚC TÍNH, chưa xác minh với cổng thanh toán.</t>
+        </is>
+      </c>
       <c r="E50" s="7" t="n"/>
       <c r="F50" s="7" t="n"/>
       <c r="G50" s="8" t="n"/>
@@ -4351,23 +4337,19 @@
     <row r="51" ht="15.5" customHeight="1">
       <c r="A51" s="18" t="inlineStr">
         <is>
-          <t>GM sau overhead (tham khảo)</t>
+          <t>GM sau phí cổng thanh toán</t>
         </is>
       </c>
       <c r="B51" s="19">
-        <f>1-'1_Cost_Job'!$B$95/$B$37</f>
-        <v>-0.45542702735317775</v>
+        <f>$B$48-$B$50</f>
+        <v>0.6700154505229284</v>
       </c>
       <c r="C51" s="15" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D51" s="16" t="inlineStr">
-        <is>
-          <t>Âm = ở quy mô hiện tại overhead chưa được phủ.</t>
-        </is>
-      </c>
+      <c r="D51" s="16" t="inlineStr"/>
       <c r="E51" s="7" t="n"/>
       <c r="F51" s="7" t="n"/>
       <c r="G51" s="8" t="n"/>
@@ -4375,111 +4357,115 @@
     <row r="52" ht="15.5" customHeight="1">
       <c r="A52" s="18" t="inlineStr">
         <is>
-          <t>Số job hoàn thành / tháng để phủ overhead</t>
-        </is>
-      </c>
-      <c r="B52" s="29">
-        <f>IF($B$37&gt;'1_Cost_Job'!$B$94,'1_Cost_Job'!$B$75/($B$37-'1_Cost_Job'!$B$94),0)</f>
-        <v>13242.208955332033</v>
+          <t>GM sau overhead (tham khảo)</t>
+        </is>
+      </c>
+      <c r="B52" s="19">
+        <f>1-'1_Cost_Job'!$B$95/$B$38</f>
+        <v>-0.45542702735317775</v>
       </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
-          <t>job</t>
+          <t>%</t>
         </is>
       </c>
       <c r="D52" s="16" t="inlineStr">
         <is>
-          <t>= Overhead / (giá − Cost/Job).</t>
+          <t>Âm = ở quy mô hiện tại overhead chưa được phủ.</t>
         </is>
       </c>
       <c r="E52" s="7" t="n"/>
       <c r="F52" s="7" t="n"/>
       <c r="G52" s="8" t="n"/>
     </row>
-    <row r="53" ht="29" customHeight="1">
+    <row r="53" ht="15.5" customHeight="1">
       <c r="A53" s="18" t="inlineStr">
         <is>
-          <t>Tương đương số khách trả phí</t>
-        </is>
-      </c>
-      <c r="B53" s="42">
-        <f>$B$52/'1_Cost_Job'!$B$22/$B$38</f>
-        <v>25.4657864525616</v>
+          <t>Số job hoàn thành / tháng để phủ overhead</t>
+        </is>
+      </c>
+      <c r="B53" s="29">
+        <f>IF($B$38&gt;'1_Cost_Job'!$B$94,'1_Cost_Job'!$B$75/($B$38-'1_Cost_Job'!$B$94),0)</f>
+        <v>13242.208955332033</v>
       </c>
       <c r="C53" s="15" t="inlineStr">
         <is>
-          <t>khách</t>
+          <t>job</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>So với mục tiêu tháng 3 ở 5_90Day_Plan: chưa phủ overhead trong 90 ngày — chấp nhận được ở giai đoạn học, nhưng phải nói rõ.</t>
+          <t>= Overhead / (giá − Cost/Job).</t>
         </is>
       </c>
       <c r="E53" s="7" t="n"/>
       <c r="F53" s="7" t="n"/>
       <c r="G53" s="8" t="n"/>
     </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="3" t="inlineStr">
+    <row r="54" ht="29" customHeight="1">
+      <c r="A54" s="18" t="inlineStr">
+        <is>
+          <t>Tương đương số khách trả phí</t>
+        </is>
+      </c>
+      <c r="B54" s="42">
+        <f>$B$53/'1_Cost_Job'!$B$22/$B$39</f>
+        <v>25.4657864525616</v>
+      </c>
+      <c r="C54" s="15" t="inlineStr">
+        <is>
+          <t>khách</t>
+        </is>
+      </c>
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>So với mục tiêu tháng 3 ở 5_90Day_Plan: chưa phủ overhead trong 90 ngày — chấp nhận được ở giai đoạn học, nhưng phải nói rõ.</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="n"/>
+      <c r="F54" s="7" t="n"/>
+      <c r="G54" s="8" t="n"/>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>E. Breakeven containment — containment tối thiểu để GM ≥ mục tiêu (nghiệm đóng, không cần Goal Seek)</t>
         </is>
       </c>
-      <c r="B55" s="4" t="n"/>
-      <c r="C55" s="4" t="n"/>
-      <c r="D55" s="4" t="n"/>
-      <c r="E55" s="4" t="n"/>
-      <c r="F55" s="4" t="n"/>
-      <c r="G55" s="4" t="n"/>
-    </row>
-    <row r="56" ht="27" customHeight="1">
-      <c r="A56" s="27" t="inlineStr">
-        <is>
-          <t>Đặt F = API + Retry + Infra (cố định theo job THỬ N), h = QA nội bộ / job hoàn thành, e = chi phí xử lý tay / job escalate (chỉ Biến thể B), P = giá, g = mục tiêu GM, R = containment.</t>
-        </is>
-      </c>
+      <c r="B56" s="4" t="n"/>
+      <c r="C56" s="4" t="n"/>
+      <c r="D56" s="4" t="n"/>
+      <c r="E56" s="4" t="n"/>
+      <c r="F56" s="4" t="n"/>
+      <c r="G56" s="4" t="n"/>
     </row>
     <row r="57" ht="27" customHeight="1">
       <c r="A57" s="27" t="inlineStr">
         <is>
+          <t>Đặt F = API + Retry + Infra (cố định theo job THỬ N), h = QA nội bộ / job hoàn thành, e = chi phí xử lý tay / job escalate (chỉ Biến thể B), P = giá, g = mục tiêu GM, R = containment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="27" customHeight="1">
+      <c r="A58" s="27" t="inlineStr">
+        <is>
           <t>Biến thể A: Cost/Job(R) = F/(N·R) + h ≤ (1−g)·P  ⇒  R ≥ F / [ N · ((1−g)·P − h) ].   Biến thể B: Cost/Job(R) = (F + e·N)/(N·R) + (h − e) ≤ (1−g)·P  ⇒  R ≥ (F + e·N) / [ N · ((1−g)·P − (h − e)) ].</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="15.5" customHeight="1">
-      <c r="A58" s="18" t="inlineStr">
+    <row r="59" ht="15.5" customHeight="1">
+      <c r="A59" s="18" t="inlineStr">
         <is>
           <t>F = API + Retry + Infra / tháng</t>
         </is>
       </c>
-      <c r="B58" s="20">
+      <c r="B59" s="20">
         <f>'1_Cost_Job'!$B$79+'1_Cost_Job'!$B$80+'1_Cost_Job'!$B$81</f>
         <v>240.63600000000002</v>
       </c>
-      <c r="C58" s="15" t="inlineStr">
+      <c r="C59" s="15" t="inlineStr">
         <is>
           <t>$ / tháng</t>
-        </is>
-      </c>
-      <c r="D58" s="16" t="inlineStr"/>
-      <c r="E58" s="7" t="n"/>
-      <c r="F58" s="7" t="n"/>
-      <c r="G58" s="8" t="n"/>
-    </row>
-    <row r="59" ht="15.5" customHeight="1">
-      <c r="A59" s="18" t="inlineStr">
-        <is>
-          <t>h = QA nội bộ / job hoàn thành</t>
-        </is>
-      </c>
-      <c r="B59" s="32">
-        <f>'1_Cost_Job'!$B$68*'1_Cost_Job'!$B$69/60*'1_Cost_Job'!$B$67</f>
-        <v>0.007792207792207793</v>
-      </c>
-      <c r="C59" s="15" t="inlineStr">
-        <is>
-          <t>$ / job</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr"/>
@@ -4490,12 +4476,12 @@
     <row r="60" ht="15.5" customHeight="1">
       <c r="A60" s="18" t="inlineStr">
         <is>
-          <t>e = xử lý tay / job escalate</t>
+          <t>h = QA nội bộ / job hoàn thành</t>
         </is>
       </c>
       <c r="B60" s="32">
-        <f>'1_Cost_Job'!$B$70/60*'1_Cost_Job'!$B$67</f>
-        <v>0.25974025974025977</v>
+        <f>'1_Cost_Job'!$B$68*'1_Cost_Job'!$B$69/60*'1_Cost_Job'!$B$67</f>
+        <v>0.007792207792207793</v>
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
@@ -4510,23 +4496,19 @@
     <row r="61" ht="15.5" customHeight="1">
       <c r="A61" s="18" t="inlineStr">
         <is>
-          <t>Breakeven containment — Biến thể A</t>
-        </is>
-      </c>
-      <c r="B61" s="19">
-        <f>IF((1-$B$44)*$B$37-$B$59&lt;=0,9.99,$B$58/('1_Cost_Job'!$B$21*((1-$B$44)*$B$37-$B$59)))</f>
-        <v>0.5746102958015268</v>
+          <t>e = xử lý tay / job escalate</t>
+        </is>
+      </c>
+      <c r="B61" s="32">
+        <f>'1_Cost_Job'!$B$70/60*'1_Cost_Job'!$B$67</f>
+        <v>0.25974025974025977</v>
       </c>
       <c r="C61" s="15" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D61" s="16" t="inlineStr">
-        <is>
-          <t>9,99 = không đạt được dù containment 100%.</t>
-        </is>
-      </c>
+          <t>$ / job</t>
+        </is>
+      </c>
+      <c r="D61" s="16" t="inlineStr"/>
       <c r="E61" s="7" t="n"/>
       <c r="F61" s="7" t="n"/>
       <c r="G61" s="8" t="n"/>
@@ -4534,32 +4516,36 @@
     <row r="62" ht="15.5" customHeight="1">
       <c r="A62" s="18" t="inlineStr">
         <is>
-          <t>Breakeven containment — Biến thể B</t>
+          <t>Breakeven containment — Biến thể A</t>
         </is>
       </c>
       <c r="B62" s="19">
-        <f>IF((1-$B$44)*$B$37-($B$59-$B$60)&lt;=0,9.99,($B$58+$B$60*'1_Cost_Job'!$B$21)/('1_Cost_Job'!$B$21*((1-$B$44)*$B$37-($B$59-$B$60))))</f>
-        <v>0.9409368826179119</v>
+        <f>IF((1-$B$45)*$B$38-$B$60&lt;=0,9.99,$B$59/('1_Cost_Job'!$B$21*((1-$B$45)*$B$38-$B$60)))</f>
+        <v>0.5746102958015268</v>
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D62" s="16" t="inlineStr"/>
+      <c r="D62" s="16" t="inlineStr">
+        <is>
+          <t>9,99 = không đạt được dù containment 100%.</t>
+        </is>
+      </c>
       <c r="E62" s="7" t="n"/>
       <c r="F62" s="7" t="n"/>
       <c r="G62" s="8" t="n"/>
     </row>
     <row r="63" ht="15.5" customHeight="1">
-      <c r="A63" s="13" t="inlineStr">
-        <is>
-          <t>BREAKEVEN CONTAINMENT — biến thể đang chọn</t>
-        </is>
-      </c>
-      <c r="B63" s="17">
-        <f>IF('1_Cost_Job'!$B$8="A",$B$61,$B$62)</f>
-        <v>0.5746102958015268</v>
+      <c r="A63" s="18" t="inlineStr">
+        <is>
+          <t>Breakeven containment — Biến thể B</t>
+        </is>
+      </c>
+      <c r="B63" s="19">
+        <f>IF((1-$B$45)*$B$38-($B$60-$B$61)&lt;=0,9.99,($B$59+$B$61*'1_Cost_Job'!$B$21)/('1_Cost_Job'!$B$21*((1-$B$45)*$B$38-($B$60-$B$61))))</f>
+        <v>0.9409368826179119</v>
       </c>
       <c r="C63" s="15" t="inlineStr">
         <is>
@@ -4572,25 +4558,21 @@
       <c r="G63" s="8" t="n"/>
     </row>
     <row r="64" ht="15.5" customHeight="1">
-      <c r="A64" s="18" t="inlineStr">
-        <is>
-          <t>Containment hiện tại (ước tính — chưa có eval)</t>
-        </is>
-      </c>
-      <c r="B64" s="19">
-        <f>'1_Cost_Job'!$B$22</f>
-        <v>0.8</v>
+      <c r="A64" s="13" t="inlineStr">
+        <is>
+          <t>BREAKEVEN CONTAINMENT — biến thể đang chọn</t>
+        </is>
+      </c>
+      <c r="B64" s="17">
+        <f>IF('1_Cost_Job'!$B$8="A",$B$62,$B$63)</f>
+        <v>0.5746102958015268</v>
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D64" s="16" t="inlineStr">
-        <is>
-          <t>Liên kết từ 1_Cost_Job S2. Khi có eval, thay số ở đó.</t>
-        </is>
-      </c>
+      <c r="D64" s="16" t="inlineStr"/>
       <c r="E64" s="7" t="n"/>
       <c r="F64" s="7" t="n"/>
       <c r="G64" s="8" t="n"/>
@@ -4598,639 +4580,643 @@
     <row r="65" ht="15.5" customHeight="1">
       <c r="A65" s="18" t="inlineStr">
         <is>
-          <t>Biên an toàn</t>
+          <t>Containment hiện tại (ước tính — chưa có eval)</t>
         </is>
       </c>
       <c r="B65" s="19">
-        <f>$B$64-$B$63</f>
-        <v>0.22538970419847326</v>
+        <f>'1_Cost_Job'!$B$22</f>
+        <v>0.8</v>
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
-          <t>điểm %</t>
-        </is>
-      </c>
-      <c r="D65" s="16" t="inlineStr"/>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>Liên kết từ 1_Cost_Job S2. Khi có eval, thay số ở đó.</t>
+        </is>
+      </c>
       <c r="E65" s="7" t="n"/>
       <c r="F65" s="7" t="n"/>
       <c r="G65" s="8" t="n"/>
     </row>
-    <row r="66" ht="29" customHeight="1">
+    <row r="66" ht="15.5" customHeight="1">
       <c r="A66" s="18" t="inlineStr">
         <is>
-          <t>Đối chiếu với eval</t>
-        </is>
-      </c>
-      <c r="B66" s="22" t="str">
-        <f>IF($B$64&lt;$B$63,"✗ DƯỚI ngưỡng: mô hình lỗ ở GM mục tiêu. Hành động: tăng containment, tăng giá, hoặc đổi biến thể HITL.",IF($B$65&lt;0.1,"~ Trên ngưỡng nhưng biên an toàn &lt; 10 điểm %","✓ Trên ngưỡng với biên an toàn ≥ 10 điểm %. Lưu ý containment hiện tại là ước tính, chưa đo."))</f>
-        <v>✓ Trên ngưỡng với biên an toàn ≥ 10 điểm %. Lưu ý containment hiện tại là ước tính, chưa đo.</v>
-      </c>
-      <c r="C66" s="7" t="n"/>
-      <c r="D66" s="7" t="n"/>
+          <t>Biên an toàn</t>
+        </is>
+      </c>
+      <c r="B66" s="19">
+        <f>$B$65-$B$64</f>
+        <v>0.22538970419847326</v>
+      </c>
+      <c r="C66" s="15" t="inlineStr">
+        <is>
+          <t>điểm %</t>
+        </is>
+      </c>
+      <c r="D66" s="16" t="inlineStr"/>
       <c r="E66" s="7" t="n"/>
       <c r="F66" s="7" t="n"/>
       <c r="G66" s="8" t="n"/>
     </row>
-    <row r="68" ht="18" customHeight="1">
-      <c r="A68" s="3" t="inlineStr">
+    <row r="67" ht="29" customHeight="1">
+      <c r="A67" s="18" t="inlineStr">
+        <is>
+          <t>Đối chiếu với eval</t>
+        </is>
+      </c>
+      <c r="B67" s="22" t="str">
+        <f>IF($B$65&lt;$B$64,"✗ DƯỚI ngưỡng: mô hình lỗ ở GM mục tiêu. Hành động: tăng containment, tăng giá, hoặc đổi biến thể HITL.",IF($B$66&lt;0.1,"~ Trên ngưỡng nhưng biên an toàn &lt; 10 điểm %","✓ Trên ngưỡng với biên an toàn ≥ 10 điểm %. Lưu ý containment hiện tại là ước tính, chưa đo."))</f>
+        <v>✓ Trên ngưỡng với biên an toàn ≥ 10 điểm %. Lưu ý containment hiện tại là ước tính, chưa đo.</v>
+      </c>
+      <c r="C67" s="7" t="n"/>
+      <c r="D67" s="7" t="n"/>
+      <c r="E67" s="7" t="n"/>
+      <c r="F67" s="7" t="n"/>
+      <c r="G67" s="8" t="n"/>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="3" t="inlineStr">
         <is>
           <t>F. Bảng sensitivity — Cost/Job và GM theo containment</t>
         </is>
       </c>
-      <c r="B68" s="4" t="n"/>
-      <c r="C68" s="4" t="n"/>
-      <c r="D68" s="4" t="n"/>
-      <c r="E68" s="4" t="n"/>
-      <c r="F68" s="4" t="n"/>
-      <c r="G68" s="4" t="n"/>
-    </row>
-    <row r="69" ht="15.5" customHeight="1">
-      <c r="A69" s="35" t="inlineStr">
+      <c r="B69" s="4" t="n"/>
+      <c r="C69" s="4" t="n"/>
+      <c r="D69" s="4" t="n"/>
+      <c r="E69" s="4" t="n"/>
+      <c r="F69" s="4" t="n"/>
+      <c r="G69" s="4" t="n"/>
+    </row>
+    <row r="70" ht="15.5" customHeight="1">
+      <c r="A70" s="35" t="inlineStr">
         <is>
           <t>Kịch bản</t>
         </is>
       </c>
-      <c r="B69" s="36" t="inlineStr">
+      <c r="B70" s="36" t="inlineStr">
         <is>
           <t>Containment</t>
         </is>
       </c>
-      <c r="C69" s="36" t="inlineStr">
+      <c r="C70" s="36" t="inlineStr">
         <is>
           <t>Cost/Job A</t>
         </is>
       </c>
-      <c r="D69" s="36" t="inlineStr">
+      <c r="D70" s="36" t="inlineStr">
         <is>
           <t>GM A</t>
         </is>
       </c>
-      <c r="E69" s="36" t="inlineStr">
+      <c r="E70" s="36" t="inlineStr">
         <is>
           <t>Cost/Job B</t>
         </is>
       </c>
-      <c r="F69" s="36" t="inlineStr">
+      <c r="F70" s="36" t="inlineStr">
         <is>
           <t>GM B</t>
         </is>
       </c>
-      <c r="G69" s="36" t="inlineStr">
+      <c r="G70" s="36" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="18" t="inlineStr">
-        <is>
-          <t>Containment 50%</t>
-        </is>
-      </c>
-      <c r="B70" s="19" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C70" s="32">
-        <f>$B$58/('1_Cost_Job'!$B$21*B70)+$B$59</f>
-        <v>0.0559194077922078</v>
-      </c>
-      <c r="D70" s="19">
-        <f>1-C70/$B$37</f>
-        <v>0.5496755655671761</v>
-      </c>
-      <c r="E70" s="32">
-        <f>($B$58+$B$60*'1_Cost_Job'!$B$21)/('1_Cost_Job'!$B$21*B70)+($B$59-$B$60)</f>
-        <v>0.3156596675324675</v>
-      </c>
-      <c r="F70" s="19">
-        <f>1-E70/$B$37</f>
-        <v>-1.5420380305711983</v>
-      </c>
-      <c r="G70" s="16" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="18" t="inlineStr">
         <is>
-          <t>Containment 60%</t>
+          <t>Containment 50%</t>
         </is>
       </c>
       <c r="B71" s="19" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="C71" s="32">
-        <f>$B$58/('1_Cost_Job'!$B$21*B71)+$B$59</f>
-        <v>0.0478982077922078</v>
+        <f>$B$59/('1_Cost_Job'!$B$21*B71)+$B$60</f>
+        <v>0.0559194077922078</v>
       </c>
       <c r="D71" s="19">
-        <f>1-C71/$B$37</f>
-        <v>0.6142710699919549</v>
+        <f>1-C71/$B$38</f>
+        <v>0.5496755655671761</v>
       </c>
       <c r="E71" s="32">
-        <f>($B$58+$B$60*'1_Cost_Job'!$B$21)/('1_Cost_Job'!$B$21*B71)+($B$59-$B$60)</f>
-        <v>0.22105838095238095</v>
+        <f>($B$59+$B$61*'1_Cost_Job'!$B$21)/('1_Cost_Job'!$B$21*B71)+($B$60-$B$61)</f>
+        <v>0.3156596675324675</v>
       </c>
       <c r="F71" s="19">
-        <f>1-E71/$B$37</f>
-        <v>-0.7802046607669615</v>
+        <f>1-E71/$B$38</f>
+        <v>-1.5420380305711983</v>
       </c>
       <c r="G71" s="16" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="18" t="inlineStr">
         <is>
-          <t>Containment 70%</t>
+          <t>Containment 60%</t>
         </is>
       </c>
       <c r="B72" s="19" t="n">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="C72" s="32">
-        <f>$B$58/('1_Cost_Job'!$B$21*B72)+$B$59</f>
-        <v>0.042168779220779225</v>
+        <f>$B$59/('1_Cost_Job'!$B$21*B72)+$B$60</f>
+        <v>0.0478982077922078</v>
       </c>
       <c r="D72" s="19">
-        <f>1-C72/$B$37</f>
-        <v>0.6604107160096541</v>
+        <f>1-C72/$B$38</f>
+        <v>0.6142710699919549</v>
       </c>
       <c r="E72" s="32">
-        <f>($B$58+$B$60*'1_Cost_Job'!$B$21)/('1_Cost_Job'!$B$21*B72)+($B$59-$B$60)</f>
-        <v>0.15348603339517625</v>
+        <f>($B$59+$B$61*'1_Cost_Job'!$B$21)/('1_Cost_Job'!$B$21*B72)+($B$60-$B$61)</f>
+        <v>0.22105838095238095</v>
       </c>
       <c r="F72" s="19">
-        <f>1-E72/$B$37</f>
-        <v>-0.23603796804964938</v>
+        <f>1-E72/$B$38</f>
+        <v>-0.7802046607669615</v>
       </c>
       <c r="G72" s="16" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="18" t="inlineStr">
         <is>
-          <t>Containment 80%</t>
+          <t>Containment 70%</t>
         </is>
       </c>
       <c r="B73" s="19" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="C73" s="32">
-        <f>$B$58/('1_Cost_Job'!$B$21*B73)+$B$59</f>
-        <v>0.0378717077922078</v>
+        <f>$B$59/('1_Cost_Job'!$B$21*B73)+$B$60</f>
+        <v>0.042168779220779225</v>
       </c>
       <c r="D73" s="19">
-        <f>1-C73/$B$37</f>
-        <v>0.6950154505229283</v>
+        <f>1-C73/$B$38</f>
+        <v>0.6604107160096541</v>
       </c>
       <c r="E73" s="32">
-        <f>($B$58+$B$60*'1_Cost_Job'!$B$21)/('1_Cost_Job'!$B$21*B73)+($B$59-$B$60)</f>
-        <v>0.10280677272727273</v>
+        <f>($B$59+$B$61*'1_Cost_Job'!$B$21)/('1_Cost_Job'!$B$21*B73)+($B$60-$B$61)</f>
+        <v>0.15348603339517625</v>
       </c>
       <c r="F73" s="19">
-        <f>1-E73/$B$37</f>
-        <v>0.1720870514883347</v>
+        <f>1-E73/$B$38</f>
+        <v>-0.23603796804964938</v>
       </c>
       <c r="G73" s="16" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="18" t="inlineStr">
         <is>
+          <t>Containment 80%</t>
+        </is>
+      </c>
+      <c r="B74" s="19" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C74" s="32">
+        <f>$B$59/('1_Cost_Job'!$B$21*B74)+$B$60</f>
+        <v>0.0378717077922078</v>
+      </c>
+      <c r="D74" s="19">
+        <f>1-C74/$B$38</f>
+        <v>0.6950154505229283</v>
+      </c>
+      <c r="E74" s="32">
+        <f>($B$59+$B$61*'1_Cost_Job'!$B$21)/('1_Cost_Job'!$B$21*B74)+($B$60-$B$61)</f>
+        <v>0.10280677272727273</v>
+      </c>
+      <c r="F74" s="19">
+        <f>1-E74/$B$38</f>
+        <v>0.1720870514883347</v>
+      </c>
+      <c r="G74" s="16" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="18" t="inlineStr">
+        <is>
           <t>Containment 90%</t>
         </is>
       </c>
-      <c r="B74" s="19" t="n">
+      <c r="B75" s="19" t="n">
         <v>0.9</v>
       </c>
-      <c r="C74" s="32">
-        <f>$B$58/('1_Cost_Job'!$B$21*B74)+$B$59</f>
+      <c r="C75" s="32">
+        <f>$B$59/('1_Cost_Job'!$B$21*B75)+$B$60</f>
         <v>0.03452954112554113</v>
       </c>
-      <c r="D74" s="19">
-        <f>1-C74/$B$37</f>
+      <c r="D75" s="19">
+        <f>1-C75/$B$38</f>
         <v>0.7219302440332529</v>
       </c>
-      <c r="E74" s="32">
-        <f>($B$58+$B$60*'1_Cost_Job'!$B$21)/('1_Cost_Job'!$B$21*B74)+($B$59-$B$60)</f>
+      <c r="E75" s="32">
+        <f>($B$59+$B$61*'1_Cost_Job'!$B$21)/('1_Cost_Job'!$B$21*B75)+($B$60-$B$61)</f>
         <v>0.06338956998557</v>
       </c>
-      <c r="F74" s="19">
-        <f>1-E74/$B$37</f>
+      <c r="F75" s="19">
+        <f>1-E75/$B$38</f>
         <v>0.4895176222401001</v>
       </c>
-      <c r="G74" s="16" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="13" t="inlineStr">
+      <c r="G75" s="16" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="13" t="inlineStr">
         <is>
           <t>Hiện tại (ước tính)</t>
         </is>
       </c>
-      <c r="B75" s="19">
+      <c r="B76" s="19">
         <f>'1_Cost_Job'!$B$22</f>
         <v>0.8</v>
       </c>
-      <c r="C75" s="32">
-        <f>$B$58/('1_Cost_Job'!$B$21*B75)+$B$59</f>
+      <c r="C76" s="32">
+        <f>$B$59/('1_Cost_Job'!$B$21*B76)+$B$60</f>
         <v>0.0378717077922078</v>
       </c>
-      <c r="D75" s="19">
-        <f>1-C75/$B$37</f>
+      <c r="D76" s="19">
+        <f>1-C76/$B$38</f>
         <v>0.6950154505229283</v>
       </c>
-      <c r="E75" s="32">
-        <f>($B$58+$B$60*'1_Cost_Job'!$B$21)/('1_Cost_Job'!$B$21*B75)+($B$59-$B$60)</f>
+      <c r="E76" s="32">
+        <f>($B$59+$B$61*'1_Cost_Job'!$B$21)/('1_Cost_Job'!$B$21*B76)+($B$60-$B$61)</f>
         <v>0.10280677272727273</v>
       </c>
-      <c r="F75" s="19">
-        <f>1-E75/$B$37</f>
+      <c r="F76" s="19">
+        <f>1-E76/$B$38</f>
         <v>0.1720870514883347</v>
       </c>
-      <c r="G75" s="16" t="inlineStr">
+      <c r="G76" s="16" t="inlineStr">
         <is>
           <t>Khớp Tab 1 (kiểm chứng chéo)</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="14.5" customHeight="1">
-      <c r="A76" s="27" t="inlineStr">
+    <row r="77" ht="14.5" customHeight="1">
+      <c r="A77" s="27" t="inlineStr">
         <is>
           <t>Ô xanh = GM ≥ mục tiêu · vàng = 50–60% · đỏ = &lt; 50% · cam = &gt; 85% (nghi quên chi phí).</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="18" customHeight="1">
-      <c r="A78" s="3" t="inlineStr">
+    <row r="79" ht="18" customHeight="1">
+      <c r="A79" s="3" t="inlineStr">
         <is>
           <t>G. Stress test giá — đổi model LLM (Prompt 4.7.1 mục 4: giá nào có thể đổi trong 6 tháng?)</t>
         </is>
       </c>
-      <c r="B78" s="4" t="n"/>
-      <c r="C78" s="4" t="n"/>
-      <c r="D78" s="4" t="n"/>
-      <c r="E78" s="4" t="n"/>
-      <c r="F78" s="4" t="n"/>
-      <c r="G78" s="4" t="n"/>
-    </row>
-    <row r="79" ht="29" customHeight="1">
-      <c r="A79" s="35" t="inlineStr">
+      <c r="B79" s="4" t="n"/>
+      <c r="C79" s="4" t="n"/>
+      <c r="D79" s="4" t="n"/>
+      <c r="E79" s="4" t="n"/>
+      <c r="F79" s="4" t="n"/>
+      <c r="G79" s="4" t="n"/>
+    </row>
+    <row r="80" ht="29" customHeight="1">
+      <c r="A80" s="35" t="inlineStr">
         <is>
           <t>Model LLM (giá ở 6_Benchmarks)</t>
         </is>
       </c>
-      <c r="B79" s="36" t="inlineStr">
+      <c r="B80" s="36" t="inlineStr">
         <is>
           <t>LLM $ / job</t>
         </is>
       </c>
-      <c r="C79" s="36" t="inlineStr">
+      <c r="C80" s="36" t="inlineStr">
         <is>
           <t>Cost/Job</t>
         </is>
       </c>
-      <c r="D79" s="36" t="inlineStr">
+      <c r="D80" s="36" t="inlineStr">
         <is>
           <t>Giá sàn 3×</t>
         </is>
       </c>
-      <c r="E79" s="36" t="inlineStr">
+      <c r="E80" s="36" t="inlineStr">
         <is>
           <t>GM @ giá đề xuất</t>
         </is>
       </c>
-      <c r="F79" s="36" t="inlineStr">
+      <c r="F80" s="36" t="inlineStr">
         <is>
           <t>GM ≥ 60%?</t>
         </is>
       </c>
-      <c r="G79" s="36" t="inlineStr">
+      <c r="G80" s="36" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="42.5" customHeight="1">
-      <c r="A80" s="13" t="inlineStr">
+    <row r="81" ht="42.5" customHeight="1">
+      <c r="A81" s="13" t="inlineStr">
         <is>
           <t>Claude Haiku 5.5</t>
-        </is>
-      </c>
-      <c r="B80" s="32">
-        <f>('1_Cost_Job'!$B$33*(INDEX('6_Benchmarks'!$C$6:$C$12,MATCH($A80,'6_Benchmarks'!$A$6:$A$12,0))+('1_Cost_Job'!$B$37-1)*INDEX('6_Benchmarks'!$D$6:$D$12,MATCH($A80,'6_Benchmarks'!$A$6:$A$12,0)))/'1_Cost_Job'!$B$36+'1_Cost_Job'!$B$32*'1_Cost_Job'!$B$34*INDEX('6_Benchmarks'!$B$6:$B$12,MATCH($A80,'6_Benchmarks'!$A$6:$A$12,0))+'1_Cost_Job'!$B$32*'1_Cost_Job'!$B$35*INDEX('6_Benchmarks'!$E$6:$E$12,MATCH($A80,'6_Benchmarks'!$A$6:$A$12,0)))/1000000</f>
-        <v>0.000823</v>
-      </c>
-      <c r="C80" s="32">
-        <f>('1_Cost_Job'!$B$21*(B80+'1_Cost_Job'!$B$51)*(1+'1_Cost_Job'!$B$61)+'1_Cost_Job'!$B$81+'1_Cost_Job'!$B$97)/'1_Cost_Job'!$B$23</f>
-        <v>0.01826797029220779</v>
-      </c>
-      <c r="D80" s="32">
-        <f>$B$6*C80</f>
-        <v>0.05480391087662337</v>
-      </c>
-      <c r="E80" s="19">
-        <f>1-C80/$B$37</f>
-        <v>0.8528862569388576</v>
-      </c>
-      <c r="F80" s="43" t="str">
-        <f>IF(AND(E80&gt;=$B$44,E80&lt;=0.85),"✓",IF(E80&gt;0.85,"~ &gt;85%","✗"))</f>
-        <v>~ &gt;85%</v>
-      </c>
-      <c r="G80" s="16" t="inlineStr">
-        <is>
-          <t>Rẻ hơn ~19× token nhưng chất lượng hạch toán CHƯA kiểm chứng; khi đó GM &gt; 85% → phải rà lại chi phí.</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="15.5" customHeight="1">
-      <c r="A81" s="13" t="inlineStr">
-        <is>
-          <t>Claude Haiku 4.5</t>
         </is>
       </c>
       <c r="B81" s="32">
         <f>('1_Cost_Job'!$B$33*(INDEX('6_Benchmarks'!$C$6:$C$12,MATCH($A81,'6_Benchmarks'!$A$6:$A$12,0))+('1_Cost_Job'!$B$37-1)*INDEX('6_Benchmarks'!$D$6:$D$12,MATCH($A81,'6_Benchmarks'!$A$6:$A$12,0)))/'1_Cost_Job'!$B$36+'1_Cost_Job'!$B$32*'1_Cost_Job'!$B$34*INDEX('6_Benchmarks'!$B$6:$B$12,MATCH($A81,'6_Benchmarks'!$A$6:$A$12,0))+'1_Cost_Job'!$B$32*'1_Cost_Job'!$B$35*INDEX('6_Benchmarks'!$E$6:$E$12,MATCH($A81,'6_Benchmarks'!$A$6:$A$12,0)))/1000000</f>
-        <v>0.00823</v>
+        <v>0.000823</v>
       </c>
       <c r="C81" s="32">
         <f>('1_Cost_Job'!$B$21*(B81+'1_Cost_Job'!$B$51)*(1+'1_Cost_Job'!$B$61)+'1_Cost_Job'!$B$81+'1_Cost_Job'!$B$97)/'1_Cost_Job'!$B$23</f>
-        <v>0.028174832792207796</v>
+        <v>0.01826797029220779</v>
       </c>
       <c r="D81" s="32">
         <f>$B$6*C81</f>
-        <v>0.08452449837662339</v>
+        <v>0.05480391087662337</v>
       </c>
       <c r="E81" s="19">
-        <f>1-C81/$B$37</f>
-        <v>0.7731053288415124</v>
+        <f>1-C81/$B$38</f>
+        <v>0.8528862569388576</v>
       </c>
       <c r="F81" s="43" t="str">
-        <f>IF(AND(E81&gt;=$B$44,E81&lt;=0.85),"✓",IF(E81&gt;0.85,"~ &gt;85%","✗"))</f>
-        <v>✓</v>
-      </c>
-      <c r="G81" s="16" t="inlineStr"/>
+        <f>IF(AND(E81&gt;=$B$45,E81&lt;=0.85),"✓",IF(E81&gt;0.85,"~ &gt;85%","✗"))</f>
+        <v>~ &gt;85%</v>
+      </c>
+      <c r="G81" s="16" t="inlineStr">
+        <is>
+          <t>Rẻ hơn ~19× token nhưng chất lượng hạch toán CHƯA kiểm chứng; khi đó GM &gt; 85% → phải rà lại chi phí.</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="15.5" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
         <is>
-          <t>Claude Sonnet 5.5</t>
+          <t>Claude Haiku 4.5</t>
         </is>
       </c>
       <c r="B82" s="32">
         <f>('1_Cost_Job'!$B$33*(INDEX('6_Benchmarks'!$C$6:$C$12,MATCH($A82,'6_Benchmarks'!$A$6:$A$12,0))+('1_Cost_Job'!$B$37-1)*INDEX('6_Benchmarks'!$D$6:$D$12,MATCH($A82,'6_Benchmarks'!$A$6:$A$12,0)))/'1_Cost_Job'!$B$36+'1_Cost_Job'!$B$32*'1_Cost_Job'!$B$34*INDEX('6_Benchmarks'!$B$6:$B$12,MATCH($A82,'6_Benchmarks'!$A$6:$A$12,0))+'1_Cost_Job'!$B$32*'1_Cost_Job'!$B$35*INDEX('6_Benchmarks'!$E$6:$E$12,MATCH($A82,'6_Benchmarks'!$A$6:$A$12,0)))/1000000</f>
-        <v>0.01548</v>
+        <v>0.00823</v>
       </c>
       <c r="C82" s="32">
         <f>('1_Cost_Job'!$B$21*(B82+'1_Cost_Job'!$B$51)*(1+'1_Cost_Job'!$B$61)+'1_Cost_Job'!$B$81+'1_Cost_Job'!$B$97)/'1_Cost_Job'!$B$23</f>
-        <v>0.03787170779220779</v>
+        <v>0.028174832792207796</v>
       </c>
       <c r="D82" s="32">
         <f>$B$6*C82</f>
-        <v>0.11361512337662337</v>
+        <v>0.08452449837662339</v>
       </c>
       <c r="E82" s="19">
-        <f>1-C82/$B$37</f>
-        <v>0.6950154505229285</v>
+        <f>1-C82/$B$38</f>
+        <v>0.7731053288415124</v>
       </c>
       <c r="F82" s="43" t="str">
-        <f>IF(AND(E82&gt;=$B$44,E82&lt;=0.85),"✓",IF(E82&gt;0.85,"~ &gt;85%","✗"))</f>
+        <f>IF(AND(E82&gt;=$B$45,E82&lt;=0.85),"✓",IF(E82&gt;0.85,"~ &gt;85%","✗"))</f>
         <v>✓</v>
       </c>
-      <c r="G82" s="16" t="inlineStr">
-        <is>
-          <t>Base case.</t>
-        </is>
-      </c>
+      <c r="G82" s="16" t="inlineStr"/>
     </row>
     <row r="83" ht="15.5" customHeight="1">
       <c r="A83" s="13" t="inlineStr">
         <is>
-          <t>Claude Opus 5.5</t>
+          <t>Claude Sonnet 5.5</t>
         </is>
       </c>
       <c r="B83" s="32">
         <f>('1_Cost_Job'!$B$33*(INDEX('6_Benchmarks'!$C$6:$C$12,MATCH($A83,'6_Benchmarks'!$A$6:$A$12,0))+('1_Cost_Job'!$B$37-1)*INDEX('6_Benchmarks'!$D$6:$D$12,MATCH($A83,'6_Benchmarks'!$A$6:$A$12,0)))/'1_Cost_Job'!$B$36+'1_Cost_Job'!$B$32*'1_Cost_Job'!$B$34*INDEX('6_Benchmarks'!$B$6:$B$12,MATCH($A83,'6_Benchmarks'!$A$6:$A$12,0))+'1_Cost_Job'!$B$32*'1_Cost_Job'!$B$35*INDEX('6_Benchmarks'!$E$6:$E$12,MATCH($A83,'6_Benchmarks'!$A$6:$A$12,0)))/1000000</f>
-        <v>0.03096</v>
+        <v>0.01548</v>
       </c>
       <c r="C83" s="32">
         <f>('1_Cost_Job'!$B$21*(B83+'1_Cost_Job'!$B$51)*(1+'1_Cost_Job'!$B$61)+'1_Cost_Job'!$B$81+'1_Cost_Job'!$B$97)/'1_Cost_Job'!$B$23</f>
-        <v>0.0585762077922078</v>
+        <v>0.03787170779220779</v>
       </c>
       <c r="D83" s="32">
         <f>$B$6*C83</f>
+        <v>0.11361512337662337</v>
+      </c>
+      <c r="E83" s="19">
+        <f>1-C83/$B$38</f>
+        <v>0.6950154505229285</v>
+      </c>
+      <c r="F83" s="43" t="str">
+        <f>IF(AND(E83&gt;=$B$45,E83&lt;=0.85),"✓",IF(E83&gt;0.85,"~ &gt;85%","✗"))</f>
+        <v>✓</v>
+      </c>
+      <c r="G83" s="16" t="inlineStr">
+        <is>
+          <t>Base case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="15.5" customHeight="1">
+      <c r="A84" s="13" t="inlineStr">
+        <is>
+          <t>Claude Opus 5.5</t>
+        </is>
+      </c>
+      <c r="B84" s="32">
+        <f>('1_Cost_Job'!$B$33*(INDEX('6_Benchmarks'!$C$6:$C$12,MATCH($A84,'6_Benchmarks'!$A$6:$A$12,0))+('1_Cost_Job'!$B$37-1)*INDEX('6_Benchmarks'!$D$6:$D$12,MATCH($A84,'6_Benchmarks'!$A$6:$A$12,0)))/'1_Cost_Job'!$B$36+'1_Cost_Job'!$B$32*'1_Cost_Job'!$B$34*INDEX('6_Benchmarks'!$B$6:$B$12,MATCH($A84,'6_Benchmarks'!$A$6:$A$12,0))+'1_Cost_Job'!$B$32*'1_Cost_Job'!$B$35*INDEX('6_Benchmarks'!$E$6:$E$12,MATCH($A84,'6_Benchmarks'!$A$6:$A$12,0)))/1000000</f>
+        <v>0.03096</v>
+      </c>
+      <c r="C84" s="32">
+        <f>('1_Cost_Job'!$B$21*(B84+'1_Cost_Job'!$B$51)*(1+'1_Cost_Job'!$B$61)+'1_Cost_Job'!$B$81+'1_Cost_Job'!$B$97)/'1_Cost_Job'!$B$23</f>
+        <v>0.0585762077922078</v>
+      </c>
+      <c r="D84" s="32">
+        <f>$B$6*C84</f>
         <v>0.1757286233766234</v>
       </c>
-      <c r="E83" s="19">
-        <f>1-C83/$B$37</f>
+      <c r="E84" s="19">
+        <f>1-C84/$B$38</f>
         <v>0.5282800965406275</v>
       </c>
-      <c r="F83" s="43" t="str">
-        <f>IF(AND(E83&gt;=$B$44,E83&lt;=0.85),"✓",IF(E83&gt;0.85,"~ &gt;85%","✗"))</f>
+      <c r="F84" s="43" t="str">
+        <f>IF(AND(E84&gt;=$B$45,E84&lt;=0.85),"✓",IF(E84&gt;0.85,"~ &gt;85%","✗"))</f>
         <v>✗</v>
       </c>
-      <c r="G83" s="16" t="inlineStr">
+      <c r="G84" s="16" t="inlineStr">
         <is>
           <t>Chỉ khi eval chứng minh cần.</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="14.5" customHeight="1">
-      <c r="A84" s="27" t="inlineStr">
+    <row r="85" ht="14.5" customHeight="1">
+      <c r="A85" s="27" t="inlineStr">
         <is>
           <t>Giá model: Anthropic, kiểm tra 13/10/2026 (không có giá khuyến mại nào trong base case). Chỉ đổi ô "Model LLM" ở 1_Cost_Job để cả mô hình chạy theo model đó.</t>
         </is>
       </c>
     </row>
-    <row r="86" ht="18" customHeight="1">
-      <c r="A86" s="3" t="inlineStr">
+    <row r="87" ht="18" customHeight="1">
+      <c r="A87" s="3" t="inlineStr">
         <is>
           <t>H. "Con số giết bạn" — sai 2× ở đâu thì mô hình gãy? (Prompt 4.7.1 mục 6)</t>
         </is>
       </c>
-      <c r="B86" s="4" t="n"/>
-      <c r="C86" s="4" t="n"/>
-      <c r="D86" s="4" t="n"/>
-      <c r="E86" s="4" t="n"/>
-      <c r="F86" s="4" t="n"/>
-      <c r="G86" s="4" t="n"/>
-    </row>
-    <row r="87" ht="15.5" customHeight="1">
-      <c r="A87" s="35" t="inlineStr">
+      <c r="B87" s="4" t="n"/>
+      <c r="C87" s="4" t="n"/>
+      <c r="D87" s="4" t="n"/>
+      <c r="E87" s="4" t="n"/>
+      <c r="F87" s="4" t="n"/>
+      <c r="G87" s="4" t="n"/>
+    </row>
+    <row r="88" ht="15.5" customHeight="1">
+      <c r="A88" s="35" t="inlineStr">
         <is>
           <t>Nếu ước tính sai 2× ở…</t>
         </is>
       </c>
-      <c r="B87" s="36" t="inlineStr">
+      <c r="B88" s="36" t="inlineStr">
         <is>
           <t>Cost/Job</t>
         </is>
       </c>
-      <c r="C87" s="36" t="inlineStr">
+      <c r="C88" s="36" t="inlineStr">
         <is>
           <t>GM</t>
         </is>
       </c>
-      <c r="D87" s="36" t="inlineStr">
+      <c r="D88" s="36" t="inlineStr">
         <is>
           <t>GM tụt (điểm %)</t>
         </is>
       </c>
-      <c r="E87" s="36" t="inlineStr"/>
-      <c r="F87" s="36" t="inlineStr"/>
-      <c r="G87" s="36" t="inlineStr">
+      <c r="E88" s="36" t="inlineStr"/>
+      <c r="F88" s="36" t="inlineStr"/>
+      <c r="G88" s="36" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="15.5" customHeight="1">
-      <c r="A88" s="18" t="inlineStr">
+    <row r="89" ht="15.5" customHeight="1">
+      <c r="A89" s="18" t="inlineStr">
         <is>
           <t>Chi phí API / token (×2)</t>
         </is>
       </c>
-      <c r="B88" s="32">
+      <c r="B89" s="32">
         <f>(2*('1_Cost_Job'!$B$79+'1_Cost_Job'!$B$80)+'1_Cost_Job'!$B$81+'1_Cost_Job'!$B$97)/'1_Cost_Job'!$B$23</f>
         <v>0.0585762077922078</v>
       </c>
-      <c r="C88" s="19">
-        <f>1-B88/$B$37</f>
+      <c r="C89" s="19">
+        <f>1-B89/$B$38</f>
         <v>0.5282800965406275</v>
       </c>
-      <c r="D88" s="19">
-        <f>$B$47-C88</f>
+      <c r="D89" s="19">
+        <f>$B$48-C89</f>
         <v>0.166735353982301</v>
       </c>
-      <c r="G88" s="16" t="inlineStr"/>
-    </row>
-    <row r="89" ht="15.5" customHeight="1">
-      <c r="A89" s="18" t="inlineStr">
+      <c r="G89" s="16" t="inlineStr"/>
+    </row>
+    <row r="90" ht="15.5" customHeight="1">
+      <c r="A90" s="18" t="inlineStr">
         <is>
           <t>Infra (×2)</t>
         </is>
       </c>
-      <c r="B89" s="32">
+      <c r="B90" s="32">
         <f>('1_Cost_Job'!$B$79+'1_Cost_Job'!$B$80+2*'1_Cost_Job'!$B$81+'1_Cost_Job'!$B$97)/'1_Cost_Job'!$B$23</f>
         <v>0.04724670779220779</v>
       </c>
-      <c r="C89" s="19">
-        <f>1-B89/$B$37</f>
+      <c r="C90" s="19">
+        <f>1-B90/$B$38</f>
         <v>0.6195176629123089</v>
       </c>
-      <c r="D89" s="19">
-        <f>$B$47-C89</f>
+      <c r="D90" s="19">
+        <f>$B$48-C90</f>
         <v>0.07549778761061954</v>
       </c>
-      <c r="G89" s="16" t="inlineStr"/>
-    </row>
-    <row r="90" ht="15.5" customHeight="1">
-      <c r="A90" s="18" t="inlineStr">
+      <c r="G90" s="16" t="inlineStr"/>
+    </row>
+    <row r="91" ht="15.5" customHeight="1">
+      <c r="A91" s="18" t="inlineStr">
         <is>
           <t>HITL (×2)</t>
         </is>
       </c>
-      <c r="B90" s="32">
+      <c r="B91" s="32">
         <f>('1_Cost_Job'!$B$79+'1_Cost_Job'!$B$80+'1_Cost_Job'!$B$81+2*'1_Cost_Job'!$B$97)/'1_Cost_Job'!$B$23</f>
         <v>0.04566391558441559</v>
       </c>
-      <c r="C90" s="19">
-        <f>1-B90/$B$37</f>
+      <c r="C91" s="19">
+        <f>1-B91/$B$38</f>
         <v>0.6322640426387771</v>
       </c>
-      <c r="D90" s="19">
-        <f>$B$47-C90</f>
+      <c r="D91" s="19">
+        <f>$B$48-C91</f>
         <v>0.06275140788415134</v>
       </c>
-      <c r="G90" s="16" t="inlineStr"/>
-    </row>
-    <row r="91" ht="29" customHeight="1">
-      <c r="A91" s="18" t="inlineStr">
+      <c r="G91" s="16" t="inlineStr"/>
+    </row>
+    <row r="92" ht="29" customHeight="1">
+      <c r="A92" s="18" t="inlineStr">
         <is>
           <t>Containment giảm một nửa</t>
         </is>
       </c>
-      <c r="B91" s="32">
-        <f>IF('1_Cost_Job'!$B$8="A",$B$58/('1_Cost_Job'!$B$21*'1_Cost_Job'!$B$22/2)+$B$59,($B$58+$B$60*'1_Cost_Job'!$B$21)/('1_Cost_Job'!$B$21*'1_Cost_Job'!$B$22/2)+($B$59-$B$60))</f>
+      <c r="B92" s="32">
+        <f>IF('1_Cost_Job'!$B$8="A",$B$59/('1_Cost_Job'!$B$21*'1_Cost_Job'!$B$22/2)+$B$60,($B$59+$B$61*'1_Cost_Job'!$B$21)/('1_Cost_Job'!$B$21*'1_Cost_Job'!$B$22/2)+($B$60-$B$61))</f>
         <v>0.0679512077922078</v>
       </c>
-      <c r="C91" s="19">
-        <f>1-B91/$B$37</f>
+      <c r="C92" s="19">
+        <f>1-B92/$B$38</f>
         <v>0.45278230893000804</v>
       </c>
-      <c r="D91" s="19">
-        <f>$B$47-C91</f>
+      <c r="D92" s="19">
+        <f>$B$48-C92</f>
         <v>0.24223314159292042</v>
       </c>
-      <c r="G91" s="16" t="inlineStr">
+      <c r="G92" s="16" t="inlineStr">
         <is>
           <t>Đây là con số duy nhất chưa đo — xem Evidence Pack.</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="13" t="inlineStr">
+    <row r="93">
+      <c r="A93" s="13" t="inlineStr">
         <is>
           <t>Con số giết bạn</t>
         </is>
       </c>
-      <c r="B92" s="9" t="str">
-        <f>INDEX(A88:A91,MATCH(MAX(D88:D91),D88:D91,0))</f>
+      <c r="B93" s="9" t="str">
+        <f>INDEX(A89:A92,MATCH(MAX(D89:D92),D89:D92,0))</f>
         <v>Containment giảm một nửa</v>
       </c>
-      <c r="C92" s="7" t="n"/>
-      <c r="D92" s="7" t="n"/>
-      <c r="E92" s="7" t="n"/>
-      <c r="F92" s="7" t="n"/>
-      <c r="G92" s="8" t="n"/>
-    </row>
-    <row r="94" ht="18" customHeight="1">
-      <c r="A94" s="3" t="inlineStr">
+      <c r="C93" s="7" t="n"/>
+      <c r="D93" s="7" t="n"/>
+      <c r="E93" s="7" t="n"/>
+      <c r="F93" s="7" t="n"/>
+      <c r="G93" s="8" t="n"/>
+    </row>
+    <row r="95" ht="18" customHeight="1">
+      <c r="A95" s="3" t="inlineStr">
         <is>
           <t>5 CON SỐ BẮT BUỘC (Trạm 3)</t>
         </is>
       </c>
-      <c r="B94" s="4" t="n"/>
-      <c r="C94" s="4" t="n"/>
-      <c r="D94" s="4" t="n"/>
-      <c r="E94" s="4" t="n"/>
-      <c r="F94" s="4" t="n"/>
-      <c r="G94" s="4" t="n"/>
-    </row>
-    <row r="95" ht="15.5" customHeight="1">
-      <c r="A95" s="13" t="inlineStr">
+      <c r="B95" s="4" t="n"/>
+      <c r="C95" s="4" t="n"/>
+      <c r="D95" s="4" t="n"/>
+      <c r="E95" s="4" t="n"/>
+      <c r="F95" s="4" t="n"/>
+      <c r="G95" s="4" t="n"/>
+    </row>
+    <row r="96" ht="15.5" customHeight="1">
+      <c r="A96" s="13" t="inlineStr">
         <is>
           <t>[ ✓ ] Cost/Job (COGS, mẫu số = job hoàn thành)</t>
         </is>
       </c>
-      <c r="B95" s="14">
+      <c r="B96" s="14">
         <f>'1_Cost_Job'!$B$94</f>
         <v>0.03787170779220779</v>
       </c>
-      <c r="C95" s="15" t="inlineStr">
+      <c r="C96" s="15" t="inlineStr">
         <is>
           <t>$ / job</t>
         </is>
       </c>
-      <c r="D95" s="16" t="inlineStr">
+      <c r="D96" s="16" t="inlineStr">
         <is>
           <t>Biến thể HITL đang chọn: xem 1_Cost_Job S0.</t>
         </is>
       </c>
-      <c r="E95" s="7" t="n"/>
-      <c r="F95" s="7" t="n"/>
-      <c r="G95" s="8" t="n"/>
-    </row>
-    <row r="96" ht="15.5" customHeight="1">
-      <c r="A96" s="13" t="inlineStr">
-        <is>
-          <t>[ ✓ ] Giá sàn (= 3 × Cost/Job)</t>
-        </is>
-      </c>
-      <c r="B96" s="14">
-        <f>$B$7</f>
-        <v>0.11361512337662337</v>
-      </c>
-      <c r="C96" s="15" t="inlineStr">
-        <is>
-          <t>$ / job</t>
-        </is>
-      </c>
-      <c r="D96" s="16" t="inlineStr"/>
       <c r="E96" s="7" t="n"/>
       <c r="F96" s="7" t="n"/>
       <c r="G96" s="8" t="n"/>
@@ -5238,23 +5224,19 @@
     <row r="97" ht="15.5" customHeight="1">
       <c r="A97" s="13" t="inlineStr">
         <is>
-          <t>[ ✓ ] Giá bán đề xuất (hiệu dụng)</t>
+          <t>[ ✓ ] Giá sàn (= 3 × Cost/Job)</t>
         </is>
       </c>
       <c r="B97" s="14">
-        <f>$B$37</f>
-        <v>0.12417582417582418</v>
+        <f>$B$7</f>
+        <v>0.11361512337662337</v>
       </c>
       <c r="C97" s="15" t="inlineStr">
         <is>
           <t>$ / job</t>
         </is>
       </c>
-      <c r="D97" s="16" t="inlineStr">
-        <is>
-          <t>Hybrid, chi tiết ở mục C.</t>
-        </is>
-      </c>
+      <c r="D97" s="16" t="inlineStr"/>
       <c r="E97" s="7" t="n"/>
       <c r="F97" s="7" t="n"/>
       <c r="G97" s="8" t="n"/>
@@ -5262,19 +5244,23 @@
     <row r="98" ht="15.5" customHeight="1">
       <c r="A98" s="13" t="inlineStr">
         <is>
-          <t>[ ✓ ] Gross Margin (mục tiêu ≥ 60%)</t>
-        </is>
-      </c>
-      <c r="B98" s="17">
-        <f>$B$47</f>
-        <v>0.6950154505229285</v>
+          <t>[ ✓ ] Giá bán đề xuất (hiệu dụng)</t>
+        </is>
+      </c>
+      <c r="B98" s="14">
+        <f>$B$38</f>
+        <v>0.12417582417582418</v>
       </c>
       <c r="C98" s="15" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D98" s="16" t="inlineStr"/>
+          <t>$ / job</t>
+        </is>
+      </c>
+      <c r="D98" s="16" t="inlineStr">
+        <is>
+          <t>Hybrid, chi tiết ở mục C.</t>
+        </is>
+      </c>
       <c r="E98" s="7" t="n"/>
       <c r="F98" s="7" t="n"/>
       <c r="G98" s="8" t="n"/>
@@ -5282,57 +5268,76 @@
     <row r="99" ht="15.5" customHeight="1">
       <c r="A99" s="13" t="inlineStr">
         <is>
-          <t>[ ✓ ] Breakeven containment</t>
+          <t>[ ✓ ] Gross Margin (mục tiêu ≥ 60%)</t>
         </is>
       </c>
       <c r="B99" s="17">
-        <f>$B$63</f>
-        <v>0.5746102958015268</v>
+        <f>$B$48</f>
+        <v>0.6950154505229285</v>
       </c>
       <c r="C99" s="15" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D99" s="16" t="inlineStr">
-        <is>
-          <t>So với eval hiện tại (ước tính, chưa đo): xem ô bên dưới.</t>
-        </is>
-      </c>
+      <c r="D99" s="16" t="inlineStr"/>
       <c r="E99" s="7" t="n"/>
       <c r="F99" s="7" t="n"/>
       <c r="G99" s="8" t="n"/>
     </row>
     <row r="100" ht="15.5" customHeight="1">
-      <c r="A100" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      so với eval hiện tại</t>
-        </is>
-      </c>
-      <c r="B100" s="19">
+      <c r="A100" s="13" t="inlineStr">
+        <is>
+          <t>[ ✓ ] Breakeven containment</t>
+        </is>
+      </c>
+      <c r="B100" s="17">
         <f>$B$64</f>
-        <v>0.8</v>
+        <v>0.5746102958015268</v>
       </c>
       <c r="C100" s="15" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D100" s="16" t="inlineStr"/>
+      <c r="D100" s="16" t="inlineStr">
+        <is>
+          <t>So với eval hiện tại (ước tính, chưa đo): xem ô bên dưới.</t>
+        </is>
+      </c>
       <c r="E100" s="7" t="n"/>
       <c r="F100" s="7" t="n"/>
       <c r="G100" s="8" t="n"/>
     </row>
+    <row r="101" ht="15.5" customHeight="1">
+      <c r="A101" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      so với eval hiện tại</t>
+        </is>
+      </c>
+      <c r="B101" s="19">
+        <f>$B$65</f>
+        <v>0.8</v>
+      </c>
+      <c r="C101" s="15" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D101" s="16" t="inlineStr"/>
+      <c r="E101" s="7" t="n"/>
+      <c r="F101" s="7" t="n"/>
+      <c r="G101" s="8" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="64">
+  <mergeCells count="65">
     <mergeCell ref="D18:G18"/>
-    <mergeCell ref="B48:G48"/>
+    <mergeCell ref="B42:G42"/>
     <mergeCell ref="D12:G12"/>
     <mergeCell ref="D39:G39"/>
     <mergeCell ref="D8:G8"/>
-    <mergeCell ref="D58:G58"/>
+    <mergeCell ref="B67:G67"/>
     <mergeCell ref="D24:G24"/>
-    <mergeCell ref="D30:G30"/>
     <mergeCell ref="D64:G64"/>
     <mergeCell ref="D15:G15"/>
     <mergeCell ref="D33:G33"/>
@@ -5342,22 +5347,23 @@
     <mergeCell ref="D38:G38"/>
     <mergeCell ref="D14:G14"/>
     <mergeCell ref="D23:G23"/>
-    <mergeCell ref="D26:G26"/>
+    <mergeCell ref="D54:G54"/>
+    <mergeCell ref="A58:G58"/>
     <mergeCell ref="D59:G59"/>
     <mergeCell ref="D35:G35"/>
     <mergeCell ref="D50:G50"/>
     <mergeCell ref="D20:G20"/>
-    <mergeCell ref="D44:G44"/>
+    <mergeCell ref="A77:G77"/>
     <mergeCell ref="D60:G60"/>
+    <mergeCell ref="B49:G49"/>
     <mergeCell ref="D100:G100"/>
-    <mergeCell ref="B40:G40"/>
     <mergeCell ref="D19:G19"/>
     <mergeCell ref="D34:G34"/>
     <mergeCell ref="D63:G63"/>
-    <mergeCell ref="B92:G92"/>
     <mergeCell ref="D99:G99"/>
     <mergeCell ref="D46:G46"/>
     <mergeCell ref="D22:G22"/>
+    <mergeCell ref="D40:G40"/>
     <mergeCell ref="D31:G31"/>
     <mergeCell ref="D65:G65"/>
     <mergeCell ref="D45:G45"/>
@@ -5365,171 +5371,172 @@
     <mergeCell ref="D6:G6"/>
     <mergeCell ref="D96:G96"/>
     <mergeCell ref="B41:G41"/>
+    <mergeCell ref="D101:G101"/>
     <mergeCell ref="D52:G52"/>
     <mergeCell ref="D21:G21"/>
+    <mergeCell ref="B26:G26"/>
     <mergeCell ref="D11:G11"/>
     <mergeCell ref="D13:G13"/>
     <mergeCell ref="D27:G27"/>
-    <mergeCell ref="D49:G49"/>
-    <mergeCell ref="D95:G95"/>
     <mergeCell ref="B25:G25"/>
     <mergeCell ref="D32:G32"/>
-    <mergeCell ref="A84:G84"/>
+    <mergeCell ref="A85:G85"/>
+    <mergeCell ref="D48:G48"/>
     <mergeCell ref="D17:G17"/>
     <mergeCell ref="D61:G61"/>
-    <mergeCell ref="A56:G56"/>
-    <mergeCell ref="B66:G66"/>
     <mergeCell ref="D53:G53"/>
+    <mergeCell ref="D66:G66"/>
     <mergeCell ref="D97:G97"/>
     <mergeCell ref="D47:G47"/>
     <mergeCell ref="D16:G16"/>
     <mergeCell ref="D7:G7"/>
+    <mergeCell ref="B93:G93"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A57:G57"/>
-    <mergeCell ref="A76:G76"/>
     <mergeCell ref="D37:G37"/>
+    <mergeCell ref="D28:G28"/>
     <mergeCell ref="D62:G62"/>
   </mergeCells>
-  <conditionalFormatting sqref="B40:G41">
+  <conditionalFormatting sqref="B41:G42">
     <cfRule type="expression" priority="1" dxfId="1" stopIfTrue="1">
-      <formula>LEFT(B40,1)="✓"</formula>
+      <formula>LEFT(B41,1)="✓"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="3" stopIfTrue="1">
-      <formula>LEFT(B40,1)="✗"</formula>
+      <formula>LEFT(B41,1)="✗"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2" stopIfTrue="1">
-      <formula>LEFT(B40,1)="~"</formula>
+      <formula>LEFT(B41,1)="~"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B45:B47">
+  <conditionalFormatting sqref="B46:B48">
     <cfRule type="expression" priority="4" dxfId="0" stopIfTrue="1">
-      <formula>AND(ISNUMBER(B45),B45&gt;0.85)</formula>
+      <formula>AND(ISNUMBER(B46),B46&gt;0.85)</formula>
     </cfRule>
     <cfRule type="expression" priority="5" dxfId="1" stopIfTrue="1">
-      <formula>AND(ISNUMBER(B45),B45&gt;=$B$44)</formula>
+      <formula>AND(ISNUMBER(B46),B46&gt;=$B$45)</formula>
     </cfRule>
     <cfRule type="expression" priority="6" dxfId="2" stopIfTrue="1">
-      <formula>AND(ISNUMBER(B45),B45&gt;=0.5)</formula>
+      <formula>AND(ISNUMBER(B46),B46&gt;=0.5)</formula>
     </cfRule>
     <cfRule type="expression" priority="7" dxfId="3" stopIfTrue="1">
-      <formula>AND(ISNUMBER(B45),B45&lt;0.5)</formula>
+      <formula>AND(ISNUMBER(B46),B46&lt;0.5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B48:G48">
+  <conditionalFormatting sqref="B49:G49">
     <cfRule type="expression" priority="8" dxfId="1" stopIfTrue="1">
-      <formula>LEFT(B48,1)="✓"</formula>
+      <formula>LEFT(B49,1)="✓"</formula>
     </cfRule>
     <cfRule type="expression" priority="9" dxfId="3" stopIfTrue="1">
-      <formula>LEFT(B48,1)="✗"</formula>
+      <formula>LEFT(B49,1)="✗"</formula>
     </cfRule>
     <cfRule type="expression" priority="10" dxfId="2" stopIfTrue="1">
-      <formula>LEFT(B48,1)="~"</formula>
+      <formula>LEFT(B49,1)="~"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B50">
+  <conditionalFormatting sqref="B51">
     <cfRule type="expression" priority="11" dxfId="0" stopIfTrue="1">
-      <formula>AND(ISNUMBER(B50),B50&gt;0.85)</formula>
+      <formula>AND(ISNUMBER(B51),B51&gt;0.85)</formula>
     </cfRule>
     <cfRule type="expression" priority="12" dxfId="1" stopIfTrue="1">
-      <formula>AND(ISNUMBER(B50),B50&gt;=$B$44)</formula>
+      <formula>AND(ISNUMBER(B51),B51&gt;=$B$45)</formula>
     </cfRule>
     <cfRule type="expression" priority="13" dxfId="2" stopIfTrue="1">
-      <formula>AND(ISNUMBER(B50),B50&gt;=0.5)</formula>
+      <formula>AND(ISNUMBER(B51),B51&gt;=0.5)</formula>
     </cfRule>
     <cfRule type="expression" priority="14" dxfId="3" stopIfTrue="1">
-      <formula>AND(ISNUMBER(B50),B50&lt;0.5)</formula>
+      <formula>AND(ISNUMBER(B51),B51&lt;0.5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B66:G66">
+  <conditionalFormatting sqref="B67:G67">
     <cfRule type="expression" priority="15" dxfId="1" stopIfTrue="1">
-      <formula>LEFT(B66,1)="✓"</formula>
+      <formula>LEFT(B67,1)="✓"</formula>
     </cfRule>
     <cfRule type="expression" priority="16" dxfId="3" stopIfTrue="1">
-      <formula>LEFT(B66,1)="✗"</formula>
+      <formula>LEFT(B67,1)="✗"</formula>
     </cfRule>
     <cfRule type="expression" priority="17" dxfId="2" stopIfTrue="1">
-      <formula>LEFT(B66,1)="~"</formula>
+      <formula>LEFT(B67,1)="~"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D70:D75">
+  <conditionalFormatting sqref="D71:D76">
     <cfRule type="expression" priority="18" dxfId="0" stopIfTrue="1">
-      <formula>AND(ISNUMBER(D70),D70&gt;0.85)</formula>
+      <formula>AND(ISNUMBER(D71),D71&gt;0.85)</formula>
     </cfRule>
     <cfRule type="expression" priority="19" dxfId="1" stopIfTrue="1">
-      <formula>AND(ISNUMBER(D70),D70&gt;=$B$44)</formula>
+      <formula>AND(ISNUMBER(D71),D71&gt;=$B$45)</formula>
     </cfRule>
     <cfRule type="expression" priority="20" dxfId="2" stopIfTrue="1">
-      <formula>AND(ISNUMBER(D70),D70&gt;=0.5)</formula>
+      <formula>AND(ISNUMBER(D71),D71&gt;=0.5)</formula>
     </cfRule>
     <cfRule type="expression" priority="21" dxfId="3" stopIfTrue="1">
-      <formula>AND(ISNUMBER(D70),D70&lt;0.5)</formula>
+      <formula>AND(ISNUMBER(D71),D71&lt;0.5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F70:F75">
+  <conditionalFormatting sqref="F71:F76">
     <cfRule type="expression" priority="22" dxfId="0" stopIfTrue="1">
-      <formula>AND(ISNUMBER(F70),F70&gt;0.85)</formula>
+      <formula>AND(ISNUMBER(F71),F71&gt;0.85)</formula>
     </cfRule>
     <cfRule type="expression" priority="23" dxfId="1" stopIfTrue="1">
-      <formula>AND(ISNUMBER(F70),F70&gt;=$B$44)</formula>
+      <formula>AND(ISNUMBER(F71),F71&gt;=$B$45)</formula>
     </cfRule>
     <cfRule type="expression" priority="24" dxfId="2" stopIfTrue="1">
-      <formula>AND(ISNUMBER(F70),F70&gt;=0.5)</formula>
+      <formula>AND(ISNUMBER(F71),F71&gt;=0.5)</formula>
     </cfRule>
     <cfRule type="expression" priority="25" dxfId="3" stopIfTrue="1">
-      <formula>AND(ISNUMBER(F70),F70&lt;0.5)</formula>
+      <formula>AND(ISNUMBER(F71),F71&lt;0.5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E80:E83">
+  <conditionalFormatting sqref="E81:E84">
     <cfRule type="expression" priority="26" dxfId="0" stopIfTrue="1">
-      <formula>AND(ISNUMBER(E80),E80&gt;0.85)</formula>
+      <formula>AND(ISNUMBER(E81),E81&gt;0.85)</formula>
     </cfRule>
     <cfRule type="expression" priority="27" dxfId="1" stopIfTrue="1">
-      <formula>AND(ISNUMBER(E80),E80&gt;=$B$44)</formula>
+      <formula>AND(ISNUMBER(E81),E81&gt;=$B$45)</formula>
     </cfRule>
     <cfRule type="expression" priority="28" dxfId="2" stopIfTrue="1">
-      <formula>AND(ISNUMBER(E80),E80&gt;=0.5)</formula>
+      <formula>AND(ISNUMBER(E81),E81&gt;=0.5)</formula>
     </cfRule>
     <cfRule type="expression" priority="29" dxfId="3" stopIfTrue="1">
-      <formula>AND(ISNUMBER(E80),E80&lt;0.5)</formula>
+      <formula>AND(ISNUMBER(E81),E81&lt;0.5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F80:F83">
+  <conditionalFormatting sqref="F81:F84">
     <cfRule type="expression" priority="30" dxfId="1" stopIfTrue="1">
-      <formula>LEFT(F80,1)="✓"</formula>
+      <formula>LEFT(F81,1)="✓"</formula>
     </cfRule>
     <cfRule type="expression" priority="31" dxfId="3" stopIfTrue="1">
-      <formula>LEFT(F80,1)="✗"</formula>
+      <formula>LEFT(F81,1)="✗"</formula>
     </cfRule>
     <cfRule type="expression" priority="32" dxfId="2" stopIfTrue="1">
-      <formula>LEFT(F80,1)="~"</formula>
+      <formula>LEFT(F81,1)="~"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C88:C91">
+  <conditionalFormatting sqref="C89:C92">
     <cfRule type="expression" priority="33" dxfId="0" stopIfTrue="1">
-      <formula>AND(ISNUMBER(C88),C88&gt;0.85)</formula>
+      <formula>AND(ISNUMBER(C89),C89&gt;0.85)</formula>
     </cfRule>
     <cfRule type="expression" priority="34" dxfId="1" stopIfTrue="1">
-      <formula>AND(ISNUMBER(C88),C88&gt;=$B$44)</formula>
+      <formula>AND(ISNUMBER(C89),C89&gt;=$B$45)</formula>
     </cfRule>
     <cfRule type="expression" priority="35" dxfId="2" stopIfTrue="1">
-      <formula>AND(ISNUMBER(C88),C88&gt;=0.5)</formula>
+      <formula>AND(ISNUMBER(C89),C89&gt;=0.5)</formula>
     </cfRule>
     <cfRule type="expression" priority="36" dxfId="3" stopIfTrue="1">
-      <formula>AND(ISNUMBER(C88),C88&lt;0.5)</formula>
+      <formula>AND(ISNUMBER(C89),C89&lt;0.5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B98">
+  <conditionalFormatting sqref="B99">
     <cfRule type="expression" priority="37" dxfId="0" stopIfTrue="1">
-      <formula>AND(ISNUMBER(B98),B98&gt;0.85)</formula>
+      <formula>AND(ISNUMBER(B99),B99&gt;0.85)</formula>
     </cfRule>
     <cfRule type="expression" priority="38" dxfId="1" stopIfTrue="1">
-      <formula>AND(ISNUMBER(B98),B98&gt;=$B$44)</formula>
+      <formula>AND(ISNUMBER(B99),B99&gt;=$B$45)</formula>
     </cfRule>
     <cfRule type="expression" priority="39" dxfId="2" stopIfTrue="1">
-      <formula>AND(ISNUMBER(B98),B98&gt;=0.5)</formula>
+      <formula>AND(ISNUMBER(B99),B99&gt;=0.5)</formula>
     </cfRule>
     <cfRule type="expression" priority="40" dxfId="3" stopIfTrue="1">
-      <formula>AND(ISNUMBER(B98),B98&lt;0.5)</formula>
+      <formula>AND(ISNUMBER(B99),B99&lt;0.5)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -5921,7 +5928,7 @@
       <c r="F26" s="4" t="n"/>
       <c r="G26" s="4" t="n"/>
     </row>
-    <row r="27" ht="29" customHeight="1">
+    <row r="27" ht="15.5" customHeight="1">
       <c r="A27" s="18" t="inlineStr">
         <is>
           <t>1. Thói quen chi trả của thị trường</t>
@@ -5929,7 +5936,7 @@
       </c>
       <c r="B27" s="25" t="inlineStr">
         <is>
-          <t>SME Việt Nam quen trả theo gói tháng cố định hoặc theo số lượng chứng từ (phần mềm kế toán, dịch vụ kế toán thuê ngoài) hơn là theo kết quả.</t>
+          <t>SME Việt Nam quen trả theo gói tháng hoặc theo số chứng từ, ít khi trả theo kết quả.</t>
         </is>
       </c>
       <c r="C27" s="7" t="n"/>
@@ -5946,7 +5953,7 @@
       </c>
       <c r="B28" s="25" t="inlineStr">
         <is>
-          <t>Khách muốn biết trước hóa đơn tháng: phí nền cho phép dự toán, chỉ phần vượt gói biến động. Usage thuần làm khách sợ vượt trần vào kỳ quyết toán.</t>
+          <t>Chủ doanh nghiệp muốn biết trước tháng này trả bao nhiêu. Phí nền cố định giúp họ dự toán, chỉ phần vượt gói mới thay đổi.</t>
         </is>
       </c>
       <c r="C28" s="7" t="n"/>
@@ -5955,7 +5962,7 @@
       <c r="F28" s="7" t="n"/>
       <c r="G28" s="8" t="n"/>
     </row>
-    <row r="29" ht="29" customHeight="1">
+    <row r="29" ht="15.5" customHeight="1">
       <c r="A29" s="18" t="inlineStr">
         <is>
           <t>3. Ai chịu chi phí inference</t>
@@ -5963,7 +5970,7 @@
       </c>
       <c r="B29" s="25" t="inlineStr">
         <is>
-          <t>Bạn chịu chi phí token; Hybrid giữ doanh thu tối thiểu phủ COGS dù khách ít dùng, và Cost/Job biến động theo volume được trả lại qua phần vượt gói.</t>
+          <t>Tôi chịu tiền token. Phí nền giúp tôi vẫn thu đủ bù chi phí kể cả khi khách ít dùng.</t>
         </is>
       </c>
       <c r="C29" s="7" t="n"/>
@@ -6073,16 +6080,15 @@
       <c r="F37" s="4" t="n"/>
       <c r="G37" s="4" t="n"/>
     </row>
-    <row r="38" ht="15.5" customHeight="1">
+    <row r="38" ht="29" customHeight="1">
       <c r="A38" s="18" t="inlineStr">
         <is>
           <t>1. Tôi chọn đơn vị nào?</t>
         </is>
       </c>
-      <c r="B38" s="25" t="inlineStr">
-        <is>
-          <t>Hybrid: phí nền theo gói tháng + phí theo hóa đơn hoàn thành vượt gói.</t>
-        </is>
+      <c r="B38" s="22" t="str">
+        <f>"Tôi chọn Hybrid: phí nền theo tháng (có sẵn "&amp;'2_Pricing'!$B$32&amp;" hóa đơn) cộng phí theo từng hóa đơn xử lý xong vượt gói."</f>
+        <v>Tôi chọn Hybrid: phí nền theo tháng (có sẵn 350 hóa đơn) cộng phí theo từng hóa đơn xử lý xong vượt gói.</v>
       </c>
       <c r="C38" s="7" t="n"/>
       <c r="D38" s="7" t="n"/>
@@ -6090,15 +6096,15 @@
       <c r="F38" s="7" t="n"/>
       <c r="G38" s="8" t="n"/>
     </row>
-    <row r="39" ht="29" customHeight="1">
+    <row r="39" ht="56" customHeight="1">
       <c r="A39" s="18" t="inlineStr">
         <is>
           <t>2. Attribution và Autonomy của tôi ở mức nào — bằng chứng gì?</t>
         </is>
       </c>
       <c r="B39" s="22" t="str">
-        <f>"Attribution "&amp;$B$11&amp;" ("&amp;ROUND($B$10,1)&amp;"/5): chưa có eval ≥ 200 mẫu và chưa có baseline của khách; Autonomy "&amp;$B$20&amp;" ("&amp;ROUND($B$19,1)&amp;"/5): containment ~"&amp;ROUND('1_Cost_Job'!$B$22*100,0)&amp;"% chỉ là ước tính, kế toán vẫn duyệt hàng loạt."</f>
-        <v>Attribution THẤP (3.2/5): chưa có eval ≥ 200 mẫu và chưa có baseline của khách; Autonomy THẤP (3.2/5): containment ~80% chỉ là ước tính, kế toán vẫn duyệt hàng loạt.</v>
+        <f>"Attribution của tôi "&amp;LOWER($B$11)&amp;" ("&amp;ROUND($B$10,1)&amp;"/5) vì chưa có bộ eval từ 200 mẫu và chưa đo được thời gian xử lý trước khi dùng AI của khách. Autonomy cũng "&amp;LOWER($B$20)&amp;" ("&amp;ROUND($B$19,1)&amp;"/5) vì AI tự xong khoảng "&amp;ROUND('1_Cost_Job'!$B$22*100,0)&amp;"% (mới là ước tính) và kế toán vẫn duyệt hàng loạt."</f>
+        <v>Attribution của tôi thấp (3.2/5) vì chưa có bộ eval từ 200 mẫu và chưa đo được thời gian xử lý trước khi dùng AI của khách. Autonomy cũng thấp (3.2/5) vì AI tự xong khoảng 80% (mới là ước tính) và kế toán vẫn duyệt hàng loạt.</v>
       </c>
       <c r="C39" s="7" t="n"/>
       <c r="D39" s="7" t="n"/>
@@ -6106,16 +6112,15 @@
       <c r="F39" s="7" t="n"/>
       <c r="G39" s="8" t="n"/>
     </row>
-    <row r="40" ht="42.5" customHeight="1">
+    <row r="40" ht="56" customHeight="1">
       <c r="A40" s="18" t="inlineStr">
         <is>
           <t>3. Nếu chọn khác gợi ý của model, lý do thị trường là gì?</t>
         </is>
       </c>
-      <c r="B40" s="25" t="inlineStr">
-        <is>
-          <t>Không chọn khác: ma trận gợi ý Seat / Hybrid và tôi chọn Hybrid. Tôi CHƯA bán Outcome vì chưa có số liệu eval làm bằng chứng Attribution; sẽ xem lại khi eval cho thấy containment đo được ≥ breakeven + 10 điểm % (5_90Day_Plan, tháng 4+).</t>
-        </is>
+      <c r="B40" s="22" t="str">
+        <f>"Ma trận gợi ý "&amp;$B$23&amp;" và tôi chọn "&amp;$B$32&amp;", nên không có chỗ lệch. Tôi chưa bán theo Outcome vì chưa có số liệu chứng minh kết quả là do AI. Khi đo được AI tự xong từ "&amp;ROUND('5_90Day_Plan'!$B$29*100,1)&amp;"% trở lên trong 2 tháng, tôi sẽ xem lại."</f>
+        <v>Ma trận gợi ý Seat / Hybrid và tôi chọn Hybrid, nên không có chỗ lệch. Tôi chưa bán theo Outcome vì chưa có số liệu chứng minh kết quả là do AI. Khi đo được AI tự xong từ 67.5% trở lên trong 2 tháng, tôi sẽ xem lại.</v>
       </c>
       <c r="C40" s="7" t="n"/>
       <c r="D40" s="7" t="n"/>
@@ -6310,7 +6315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -6356,7 +6361,7 @@
         </is>
       </c>
       <c r="B5" s="20">
-        <f>'2_Pricing'!$B$35</f>
+        <f>'2_Pricing'!$B$36</f>
         <v>64.57142857142857</v>
       </c>
       <c r="C5" s="15" t="inlineStr">
@@ -6380,7 +6385,7 @@
         </is>
       </c>
       <c r="B6" s="19">
-        <f>'2_Pricing'!$B$47</f>
+        <f>'2_Pricing'!$B$48</f>
         <v>0.6950154505229285</v>
       </c>
       <c r="C6" s="15" t="inlineStr">
@@ -7017,107 +7022,103 @@
       <c r="F38" s="7" t="n"/>
       <c r="G38" s="8" t="n"/>
     </row>
-    <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="3" t="inlineStr">
+    <row r="39" ht="69.5" customHeight="1">
+      <c r="A39" s="18" t="inlineStr">
+        <is>
+          <t>Lý do chốt kênh</t>
+        </is>
+      </c>
+      <c r="B39" s="22" t="str">
+        <f>"Tôi chọn PLG vì con số cho thấy bán qua sales không chạy được. Mỗi khách trả khoảng $"&amp;ROUND($B$5,0)&amp;"/tháng nên ngân sách CAC chỉ $"&amp;ROUND($B$9,0)&amp;". Bán qua sales rep cần "&amp;ROUND($B$18,2)&amp;" deal/người/ngày, và CAC thực khoảng $"&amp;ROUND($B$26,0)&amp;", gấp "&amp;ROUND($B$27,0)&amp;" lần ngân sách. Tôi không chọn Partner-Led vì chưa có tên đối tác nào và chưa nói chuyện với ai. PLG hợp nhất vì khách chỉ cần chuyển tiếp email hóa đơn, không phải cài thêm gì."</f>
+        <v>Tôi chọn PLG vì con số cho thấy bán qua sales không chạy được. Mỗi khách trả khoảng $65/tháng nên ngân sách CAC chỉ $539. Bán qua sales rep cần 2.58 deal/người/ngày, và CAC thực khoảng $25200, gấp 47 lần ngân sách. Tôi không chọn Partner-Led vì chưa có tên đối tác nào và chưa nói chuyện với ai. PLG hợp nhất vì khách chỉ cần chuyển tiếp email hóa đơn, không phải cài thêm gì.</v>
+      </c>
+      <c r="C39" s="7" t="n"/>
+      <c r="D39" s="7" t="n"/>
+      <c r="E39" s="7" t="n"/>
+      <c r="F39" s="7" t="n"/>
+      <c r="G39" s="8" t="n"/>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>5. Nếu rơi vào vùng không khả thi — chọn 1 trong 3 lối thoát</t>
         </is>
       </c>
-      <c r="B40" s="4" t="n"/>
-      <c r="C40" s="4" t="n"/>
-      <c r="D40" s="4" t="n"/>
-      <c r="E40" s="4" t="n"/>
-      <c r="F40" s="4" t="n"/>
-      <c r="G40" s="4" t="n"/>
-    </row>
-    <row r="41" ht="15.5" customHeight="1">
-      <c r="A41" s="18" t="inlineStr">
+      <c r="B41" s="4" t="n"/>
+      <c r="C41" s="4" t="n"/>
+      <c r="D41" s="4" t="n"/>
+      <c r="E41" s="4" t="n"/>
+      <c r="F41" s="4" t="n"/>
+      <c r="G41" s="4" t="n"/>
+    </row>
+    <row r="42" ht="15.5" customHeight="1">
+      <c r="A42" s="18" t="inlineStr">
         <is>
           <t>Lối thoát đã chọn</t>
         </is>
       </c>
-      <c r="B41" s="25" t="inlineStr">
+      <c r="B42" s="25" t="inlineStr">
         <is>
           <t>Giảm giá xuống</t>
         </is>
       </c>
-      <c r="C41" s="15" t="inlineStr">
+      <c r="C42" s="15" t="inlineStr">
         <is>
           <t>chọn</t>
         </is>
       </c>
-      <c r="D41" s="16" t="inlineStr">
+      <c r="D42" s="16" t="inlineStr">
         <is>
           <t>Giảm giá xuống / Tăng giá lên / Đi Partner-Led.</t>
         </is>
       </c>
-      <c r="E41" s="7" t="n"/>
-      <c r="F41" s="7" t="n"/>
-      <c r="G41" s="8" t="n"/>
-    </row>
-    <row r="42" ht="29" customHeight="1">
-      <c r="A42" s="18" t="inlineStr">
-        <is>
-          <t>Việc cụ thể trong 30 ngày tới</t>
-        </is>
-      </c>
-      <c r="B42" s="25" t="inlineStr">
-        <is>
-          <t>Bỏ hẳn sales rep, đơn giản hóa để khách tự mua (PLG): dựng landing + hộp thư nhận email-forward, chạy concierge test với 10 kế toán SME; dừng kênh này nếu &lt; 5 người forward hóa đơn thật trong 14 ngày.</t>
-        </is>
-      </c>
-      <c r="C42" s="7" t="n"/>
-      <c r="D42" s="7" t="n"/>
       <c r="E42" s="7" t="n"/>
       <c r="F42" s="7" t="n"/>
       <c r="G42" s="8" t="n"/>
     </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="3" t="inlineStr">
+    <row r="43" ht="29" customHeight="1">
+      <c r="A43" s="18" t="inlineStr">
+        <is>
+          <t>Việc cụ thể trong 30 ngày tới</t>
+        </is>
+      </c>
+      <c r="B43" s="25" t="inlineStr">
+        <is>
+          <t>Tôi dựng trang đăng ký và hộp thư nhận email chuyển tiếp, rồi nhờ 10 kế toán dùng thử. Nếu dưới 5 người gửi hóa đơn thật trong 14 ngày, tôi dừng và quay lại phỏng vấn.</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="n"/>
+      <c r="D43" s="7" t="n"/>
+      <c r="E43" s="7" t="n"/>
+      <c r="F43" s="7" t="n"/>
+      <c r="G43" s="8" t="n"/>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>KẾT QUẢ TRẠM 4 — các con số bắt buộc</t>
         </is>
       </c>
-      <c r="B44" s="4" t="n"/>
-      <c r="C44" s="4" t="n"/>
-      <c r="D44" s="4" t="n"/>
-      <c r="E44" s="4" t="n"/>
-      <c r="F44" s="4" t="n"/>
-      <c r="G44" s="4" t="n"/>
-    </row>
-    <row r="45" ht="15.5" customHeight="1">
-      <c r="A45" s="13" t="inlineStr">
+      <c r="B45" s="4" t="n"/>
+      <c r="C45" s="4" t="n"/>
+      <c r="D45" s="4" t="n"/>
+      <c r="E45" s="4" t="n"/>
+      <c r="F45" s="4" t="n"/>
+      <c r="G45" s="4" t="n"/>
+    </row>
+    <row r="46" ht="15.5" customHeight="1">
+      <c r="A46" s="13" t="inlineStr">
         <is>
           <t>[ ✓ ] Ngân sách CAC / khách</t>
         </is>
       </c>
-      <c r="B45" s="38">
+      <c r="B46" s="38">
         <f>$B$9</f>
         <v>538.5376862337663</v>
       </c>
-      <c r="C45" s="15" t="inlineStr">
+      <c r="C46" s="15" t="inlineStr">
         <is>
           <t>$</t>
-        </is>
-      </c>
-      <c r="D45" s="16" t="inlineStr"/>
-      <c r="E45" s="7" t="n"/>
-      <c r="F45" s="7" t="n"/>
-      <c r="G45" s="8" t="n"/>
-    </row>
-    <row r="46" ht="15.5" customHeight="1">
-      <c r="A46" s="13" t="inlineStr">
-        <is>
-          <t>[ ✓ ] Số deal / AE / ngày</t>
-        </is>
-      </c>
-      <c r="B46" s="44">
-        <f>$B$18</f>
-        <v>2.5811209439528024</v>
-      </c>
-      <c r="C46" s="15" t="inlineStr">
-        <is>
-          <t>deal</t>
         </is>
       </c>
       <c r="D46" s="16" t="inlineStr"/>
@@ -7128,16 +7129,16 @@
     <row r="47" ht="15.5" customHeight="1">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>[ ✓ ] CAC thực ước tính</t>
-        </is>
-      </c>
-      <c r="B47" s="41">
-        <f>$B$26</f>
-        <v>25200.0</v>
+          <t>[ ✓ ] Số deal / AE / ngày</t>
+        </is>
+      </c>
+      <c r="B47" s="44">
+        <f>$B$18</f>
+        <v>2.5811209439528024</v>
       </c>
       <c r="C47" s="15" t="inlineStr">
         <is>
-          <t>$</t>
+          <t>deal</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr"/>
@@ -7146,18 +7147,18 @@
       <c r="G47" s="8" t="n"/>
     </row>
     <row r="48" ht="15.5" customHeight="1">
-      <c r="A48" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">      → lệch</t>
-        </is>
-      </c>
-      <c r="B48" s="40">
-        <f>$B$27</f>
-        <v>46.793382606581936</v>
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>[ ✓ ] CAC thực ước tính</t>
+        </is>
+      </c>
+      <c r="B48" s="41">
+        <f>$B$26</f>
+        <v>25200.0</v>
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>lần</t>
+          <t>$</t>
         </is>
       </c>
       <c r="D48" s="16" t="inlineStr"/>
@@ -7165,18 +7166,22 @@
       <c r="F48" s="7" t="n"/>
       <c r="G48" s="8" t="n"/>
     </row>
-    <row r="49" ht="29" customHeight="1">
+    <row r="49" ht="15.5" customHeight="1">
       <c r="A49" s="18" t="inlineStr">
         <is>
-          <t>[ ✓ ] Kênh đã chốt</t>
-        </is>
-      </c>
-      <c r="B49" s="22" t="str">
-        <f>$B$38</f>
-        <v>PLG</v>
-      </c>
-      <c r="C49" s="7" t="n"/>
-      <c r="D49" s="7" t="n"/>
+          <t xml:space="preserve">      → lệch</t>
+        </is>
+      </c>
+      <c r="B49" s="40">
+        <f>$B$27</f>
+        <v>46.793382606581936</v>
+      </c>
+      <c r="C49" s="15" t="inlineStr">
+        <is>
+          <t>lần</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr"/>
       <c r="E49" s="7" t="n"/>
       <c r="F49" s="7" t="n"/>
       <c r="G49" s="8" t="n"/>
@@ -7184,13 +7189,12 @@
     <row r="50" ht="29" customHeight="1">
       <c r="A50" s="18" t="inlineStr">
         <is>
-          <t>[ ✓ ] Nếu Partner-Led: TÊN partner · đã nói chuyện chưa?</t>
-        </is>
-      </c>
-      <c r="B50" s="25" t="inlineStr">
-        <is>
-          <t>N/A — kênh chốt là PLG. Partner-Led để dành cho tháng 4+: chưa có tên partner nào, CHƯA nói chuyện với ai ("sẽ tích hợp các nền tảng trong ngành" = chưa có kênh).</t>
-        </is>
+          <t>[ ✓ ] Kênh đã chốt</t>
+        </is>
+      </c>
+      <c r="B50" s="22" t="str">
+        <f>$B$38</f>
+        <v>PLG</v>
       </c>
       <c r="C50" s="7" t="n"/>
       <c r="D50" s="7" t="n"/>
@@ -7198,11 +7202,27 @@
       <c r="F50" s="7" t="n"/>
       <c r="G50" s="8" t="n"/>
     </row>
+    <row r="51" ht="29" customHeight="1">
+      <c r="A51" s="18" t="inlineStr">
+        <is>
+          <t>[ ✓ ] Nếu Partner-Led: TÊN partner · đã nói chuyện chưa?</t>
+        </is>
+      </c>
+      <c r="B51" s="25" t="inlineStr">
+        <is>
+          <t>N/A — kênh chốt là PLG. Partner-Led để dành cho tháng 4+: chưa có tên partner nào, CHƯA nói chuyện với ai ("sẽ tích hợp các nền tảng trong ngành" = chưa có kênh).</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="n"/>
+      <c r="D51" s="7" t="n"/>
+      <c r="E51" s="7" t="n"/>
+      <c r="F51" s="7" t="n"/>
+      <c r="G51" s="8" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="35">
+  <mergeCells count="36">
     <mergeCell ref="D18:G18"/>
     <mergeCell ref="D9:G9"/>
-    <mergeCell ref="B42:G42"/>
     <mergeCell ref="D12:G12"/>
     <mergeCell ref="D8:G8"/>
     <mergeCell ref="D25:G25"/>
@@ -7211,6 +7231,7 @@
     <mergeCell ref="E34:G34"/>
     <mergeCell ref="D15:G15"/>
     <mergeCell ref="D5:G5"/>
+    <mergeCell ref="D42:G42"/>
     <mergeCell ref="D14:G14"/>
     <mergeCell ref="B38:G38"/>
     <mergeCell ref="B19:G19"/>
@@ -7218,15 +7239,14 @@
     <mergeCell ref="D26:G26"/>
     <mergeCell ref="E36:G36"/>
     <mergeCell ref="D20:G20"/>
-    <mergeCell ref="B49:G49"/>
     <mergeCell ref="D46:G46"/>
     <mergeCell ref="E32:G32"/>
-    <mergeCell ref="D45:G45"/>
+    <mergeCell ref="B51:G51"/>
     <mergeCell ref="D6:G6"/>
     <mergeCell ref="B50:G50"/>
     <mergeCell ref="D13:G13"/>
+    <mergeCell ref="D49:G49"/>
     <mergeCell ref="D27:G27"/>
-    <mergeCell ref="D41:G41"/>
     <mergeCell ref="D48:G48"/>
     <mergeCell ref="D17:G17"/>
     <mergeCell ref="E33:G33"/>
@@ -7235,6 +7255,8 @@
     <mergeCell ref="D7:G7"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="E35:G35"/>
+    <mergeCell ref="B43:G43"/>
+    <mergeCell ref="B39:G39"/>
   </mergeCells>
   <conditionalFormatting sqref="B19:G19">
     <cfRule type="expression" priority="1" dxfId="1" stopIfTrue="1">
@@ -7251,7 +7273,7 @@
     <dataValidation sqref="B7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"SMB,Mid-market,Enterprise"</formula1>
     </dataValidation>
-    <dataValidation sqref="B41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Giảm giá xuống,Tăng giá lên,Đi Partner-Led"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7636,7 +7658,7 @@
         </is>
       </c>
       <c r="B22" s="29">
-        <f>$B$19*'2_Pricing'!$B$38</f>
+        <f>$B$19*'2_Pricing'!$B$39</f>
         <v>9750.0</v>
       </c>
       <c r="C22" s="15" t="inlineStr">
@@ -7769,7 +7791,7 @@
         </is>
       </c>
       <c r="B29" s="19">
-        <f>'2_Pricing'!$B$63+0.1</f>
+        <f>'2_Pricing'!$B$64+0.1</f>
         <v>0.6746102958015268</v>
       </c>
       <c r="C29" s="15" t="inlineStr">
@@ -7793,7 +7815,7 @@
         </is>
       </c>
       <c r="B30" s="19">
-        <f>'2_Pricing'!$B$44</f>
+        <f>'2_Pricing'!$B$45</f>
         <v>0.6</v>
       </c>
       <c r="C30" s="15" t="inlineStr">
@@ -7970,7 +7992,7 @@
       <c r="F40" s="4" t="n"/>
       <c r="G40" s="4" t="n"/>
     </row>
-    <row r="41" ht="29" customHeight="1">
+    <row r="41" ht="42.5" customHeight="1">
       <c r="A41" s="18" t="inlineStr">
         <is>
           <t>1. AI này có hallucinate không? Nếu nó nói sai với khách của tôi thì sao?</t>
@@ -7978,7 +8000,7 @@
       </c>
       <c r="B41" s="25" t="inlineStr">
         <is>
-          <t>Có thể sai. Mỗi hóa đơn có điểm tin cậy; dưới ngưỡng thì chuyển người duyệt, và không hóa đơn nào được hạch toán khi chưa qua quy tắc kiểm tra (MST, tổng tiền, thuế). Tỷ lệ chính xác công bố từ bộ eval — CHƯA có, deadline 10/11/2026.</t>
+          <t>AI có thể sai. Hóa đơn nào AI không chắc sẽ chuyển cho kế toán duyệt, và không hóa đơn nào được hạch toán nếu chưa qua kiểm tra mã số thuế, tổng tiền và thuế. Tỷ lệ chính xác tôi sẽ công bố sau khi có bộ eval (dự kiến 10/11/2026). Hiện tôi chưa có con số đó.</t>
         </is>
       </c>
       <c r="C41" s="7" t="n"/>
@@ -7995,7 +8017,7 @@
       </c>
       <c r="B42" s="25" t="inlineStr">
         <is>
-          <t>Cam kết bằng văn bản: dữ liệu của khách không được dùng để huấn luyện model. Cần Dev 1 xác nhận điều khoản của nhà cung cấp LLM trước khi gửi khách.</t>
+          <t>Dữ liệu của khách chỉ dùng để xử lý hóa đơn cho chính họ, không dùng để huấn luyện model. Tôi sẽ ghi điều này vào hợp đồng sau khi kiểm tra điều khoản của nhà cung cấp LLM.</t>
         </is>
       </c>
       <c r="C42" s="7" t="n"/>
@@ -8012,7 +8034,7 @@
       </c>
       <c r="B43" s="25" t="inlineStr">
         <is>
-          <t>Khách xuất toàn bộ hóa đơn + bút toán dạng CSV/XML bất kỳ lúc nào; dữ liệu bị xóa sau 30 ngày khi chấm dứt hợp đồng. Cần làm tính năng xuất dữ liệu trước khi cam kết (Dev 2, deadline 30/11/2026).</t>
+          <t>Khách tải được toàn bộ hóa đơn và bút toán (CSV/XML) bất cứ lúc nào, và dữ liệu bị xóa sau 30 ngày khi hết hợp đồng. Tính năng tải dữ liệu tôi dự kiến làm xong trước 30/11/2026.</t>
         </is>
       </c>
       <c r="C43" s="7" t="n"/>

</xml_diff>